<commit_message>
Upload current DATA PENCAPAIAN and today's SO/Stock/Delivery files
Previous pencapaian upload was an earlier-in-the-day snapshot with lower
achievement figures than the current source report.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/uploads/DATA PENCAPAIAN 2026.xlsx
+++ b/uploads/DATA PENCAPAIAN 2026.xlsx
@@ -298,7 +298,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2112" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="223">
   <si>
     <t>📊  PANDUAN PENGGUNAAN — DATA PENCAPAIAN 2026</t>
   </si>
@@ -967,7 +967,7 @@
     <t>→ baris 11 (manual)</t>
   </si>
   <si>
-    <t>DATA PENCAPAIAN — GLOBAL — 24 AGUSTUS 2026</t>
+    <t>DATA PENCAPAIAN — GLOBAL — 26 AGUSTUS 2026</t>
   </si>
 </sst>
 </file>
@@ -2539,6 +2539,9 @@
     <xf numFmtId="41" fontId="47" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2611,33 +2614,6 @@
     <xf numFmtId="0" fontId="29" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2668,6 +2644,33 @@
     <xf numFmtId="0" fontId="48" fillId="37" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2681,15 +2684,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="49" fillId="37" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2713,11 +2707,17 @@
     <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="27" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3486,16 +3486,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="B1" s="234" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="234"/>
+      <c r="B1" s="235" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="235"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="235" t="s">
+      <c r="B3" s="236" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="235"/>
+      <c r="C3" s="236"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
@@ -3546,10 +3546,10 @@
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="236" t="s">
+      <c r="B11" s="237" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="236"/>
+      <c r="C11" s="237"/>
     </row>
     <row r="12" spans="2:3" ht="24" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="C3" s="75">
         <f ca="1">IF($J$5&lt;&gt;"",$J$5,MAX(0,NETWORKDAYS.INTL(MAX(TODAY(),DATE(YEAR(TODAY()),8,1)),EOMONTH(DATE(YEAR(TODAY()),8,1),0),11)-MAX(0,$J$3-$J$4)))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D3" s="76" t="s">
         <v>104</v>
@@ -3809,20 +3809,20 @@
       <c r="B10" s="72" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="293">
-        <v>122025113.198008</v>
-      </c>
-      <c r="D10" s="293">
-        <v>30987765.915591002</v>
-      </c>
-      <c r="E10" s="293">
-        <v>187321413.78949499</v>
-      </c>
-      <c r="F10" s="293">
-        <v>146701033.86000001</v>
-      </c>
-      <c r="G10" s="293">
-        <v>487035326.76309401</v>
+      <c r="C10" s="234">
+        <v>148548971.92346001</v>
+      </c>
+      <c r="D10" s="234">
+        <v>34675794.324588999</v>
+      </c>
+      <c r="E10" s="234">
+        <v>201845017.44949499</v>
+      </c>
+      <c r="F10" s="234">
+        <v>158023556.22</v>
+      </c>
+      <c r="G10" s="234">
+        <v>543093339.91754401</v>
       </c>
       <c r="H10" s="111"/>
       <c r="I10" s="111"/>
@@ -3835,20 +3835,20 @@
       <c r="B11" s="72" t="s">
         <v>216</v>
       </c>
-      <c r="C11" s="293">
-        <v>313831855.63549697</v>
-      </c>
-      <c r="D11" s="293">
-        <v>71686173.307567</v>
-      </c>
-      <c r="E11" s="293">
-        <v>107095552.073377</v>
-      </c>
-      <c r="F11" s="293">
+      <c r="C11" s="234">
+        <v>324305725.654459</v>
+      </c>
+      <c r="D11" s="234">
+        <v>74140960.586657003</v>
+      </c>
+      <c r="E11" s="234">
+        <v>111974290.83337</v>
+      </c>
+      <c r="F11" s="234">
         <v>282497104.13999999</v>
       </c>
-      <c r="G11" s="293">
-        <v>775110685.15644097</v>
+      <c r="G11" s="234">
+        <v>792918081.214486</v>
       </c>
       <c r="H11" s="111"/>
       <c r="I11" s="111"/>
@@ -3861,20 +3861,20 @@
       <c r="B12" s="72" t="s">
         <v>215</v>
       </c>
-      <c r="C12" s="293">
+      <c r="C12" s="234">
         <v>3123423.4199979999</v>
       </c>
-      <c r="D12" s="293">
+      <c r="D12" s="234">
         <v>17913431</v>
       </c>
-      <c r="E12" s="293">
-        <v>233585586.67908999</v>
-      </c>
-      <c r="F12" s="293" t="s">
-        <v>166</v>
-      </c>
-      <c r="G12" s="293">
-        <v>254622441.09908801</v>
+      <c r="E12" s="234">
+        <v>305207208.67878997</v>
+      </c>
+      <c r="F12" s="234">
+        <v>0</v>
+      </c>
+      <c r="G12" s="234">
+        <v>326244063.09878802</v>
       </c>
       <c r="H12" s="111"/>
       <c r="I12" s="111"/>
@@ -3887,20 +3887,20 @@
       <c r="B13" s="72" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="293">
-        <v>152615285.64179501</v>
-      </c>
-      <c r="D13" s="293">
-        <v>51184423.356691003</v>
-      </c>
-      <c r="E13" s="293">
-        <v>139904678.24960801</v>
-      </c>
-      <c r="F13" s="293">
-        <v>79567161.549999997</v>
-      </c>
-      <c r="G13" s="293">
-        <v>423271548.79809397</v>
+      <c r="C13" s="234">
+        <v>165127480.62579501</v>
+      </c>
+      <c r="D13" s="234">
+        <v>57055830.666670002</v>
+      </c>
+      <c r="E13" s="234">
+        <v>143153326.91960201</v>
+      </c>
+      <c r="F13" s="234">
+        <v>81188783.25</v>
+      </c>
+      <c r="G13" s="234">
+        <v>446525421.46206701</v>
       </c>
       <c r="H13" s="111"/>
       <c r="I13" s="111"/>
@@ -3913,20 +3913,20 @@
       <c r="B14" s="72" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="293">
-        <v>39176085.410832003</v>
-      </c>
-      <c r="D14" s="293">
-        <v>23676563.479958002</v>
-      </c>
-      <c r="E14" s="293">
-        <v>196901774.76942301</v>
-      </c>
-      <c r="F14" s="293">
-        <v>43760135.289999999</v>
-      </c>
-      <c r="G14" s="293">
-        <v>303514558.95021302</v>
+      <c r="C14" s="234">
+        <v>41524631.450832002</v>
+      </c>
+      <c r="D14" s="234">
+        <v>24544590.529956002</v>
+      </c>
+      <c r="E14" s="234">
+        <v>213680964.269348</v>
+      </c>
+      <c r="F14" s="234">
+        <v>46246621.840000004</v>
+      </c>
+      <c r="G14" s="234">
+        <v>325996808.09013599</v>
       </c>
       <c r="H14" s="111"/>
       <c r="I14" s="111"/>
@@ -3939,20 +3939,20 @@
       <c r="B15" s="81" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="293">
-        <v>687162604.17452097</v>
-      </c>
-      <c r="D15" s="293">
-        <v>25975566.479871999</v>
-      </c>
-      <c r="E15" s="293">
-        <v>136407063.156075</v>
-      </c>
-      <c r="F15" s="293">
-        <v>336341085.36982101</v>
-      </c>
-      <c r="G15" s="293">
-        <v>1185886319.180289</v>
+      <c r="C15" s="234">
+        <v>707734634.90601301</v>
+      </c>
+      <c r="D15" s="234">
+        <v>27756665.599851999</v>
+      </c>
+      <c r="E15" s="234">
+        <v>154753955.22001499</v>
+      </c>
+      <c r="F15" s="234">
+        <v>382338202.54978102</v>
+      </c>
+      <c r="G15" s="234">
+        <v>1272583458.275661</v>
       </c>
       <c r="H15" s="111"/>
       <c r="I15" s="111"/>
@@ -3965,20 +3965,20 @@
       <c r="B16" s="72" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="293">
-        <v>371145542.77906501</v>
-      </c>
-      <c r="D16" s="293">
+      <c r="C16" s="234">
+        <v>437919164.53906399</v>
+      </c>
+      <c r="D16" s="234">
         <v>1085666.664998</v>
       </c>
-      <c r="E16" s="293">
-        <v>97949554.359935001</v>
-      </c>
-      <c r="F16" s="293">
+      <c r="E16" s="234">
+        <v>97990094.889935002</v>
+      </c>
+      <c r="F16" s="234">
         <v>14702973.119999999</v>
       </c>
-      <c r="G16" s="293">
-        <v>484883736.923998</v>
+      <c r="G16" s="234">
+        <v>551697899.21399701</v>
       </c>
       <c r="H16" s="111"/>
       <c r="I16" s="111"/>
@@ -3991,20 +3991,20 @@
       <c r="B17" s="72" t="s">
         <v>120</v>
       </c>
-      <c r="C17" s="293">
-        <v>584747098.20811999</v>
-      </c>
-      <c r="D17" s="293">
-        <v>68513920.019765005</v>
-      </c>
-      <c r="E17" s="293">
-        <v>285862027.34951901</v>
-      </c>
-      <c r="F17" s="293">
-        <v>1300038656.6399341</v>
-      </c>
-      <c r="G17" s="293">
-        <v>2239161702.2173381</v>
+      <c r="C17" s="234">
+        <v>611345406.22811997</v>
+      </c>
+      <c r="D17" s="234">
+        <v>74143784.859764993</v>
+      </c>
+      <c r="E17" s="234">
+        <v>307286171.54949898</v>
+      </c>
+      <c r="F17" s="234">
+        <v>1342211628.6399341</v>
+      </c>
+      <c r="G17" s="234">
+        <v>2334986991.277318</v>
       </c>
       <c r="H17" s="111"/>
       <c r="I17" s="111"/>
@@ -4017,20 +4017,20 @@
       <c r="B18" s="72" t="s">
         <v>122</v>
       </c>
-      <c r="C18" s="293">
-        <v>97668278.243663996</v>
-      </c>
-      <c r="D18" s="293">
-        <v>10898698.12992</v>
-      </c>
-      <c r="E18" s="293">
-        <v>77051176.078759998</v>
-      </c>
-      <c r="F18" s="293">
+      <c r="C18" s="234">
+        <v>102129134.163663</v>
+      </c>
+      <c r="D18" s="234">
+        <v>12358157.569896</v>
+      </c>
+      <c r="E18" s="234">
+        <v>110696937.35874</v>
+      </c>
+      <c r="F18" s="234">
         <v>34412433.137999997</v>
       </c>
-      <c r="G18" s="293">
-        <v>220030585.59034401</v>
+      <c r="G18" s="234">
+        <v>259596662.230299</v>
       </c>
       <c r="H18" s="111"/>
       <c r="I18" s="111"/>
@@ -4043,20 +4043,20 @@
       <c r="B19" s="72" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="293">
+      <c r="C19" s="234">
         <v>12329000</v>
       </c>
-      <c r="D19" s="293">
+      <c r="D19" s="234">
         <v>103268962.47079</v>
       </c>
-      <c r="E19" s="293">
+      <c r="E19" s="234">
         <v>37754395.5</v>
       </c>
-      <c r="F19" s="293">
-        <v>79686488.140000001</v>
-      </c>
-      <c r="G19" s="293">
-        <v>233038846.11079001</v>
+      <c r="F19" s="234">
+        <v>84291893.659999996</v>
+      </c>
+      <c r="G19" s="234">
+        <v>237644251.63079</v>
       </c>
       <c r="H19" s="111"/>
       <c r="I19" s="111"/>
@@ -4069,20 +4069,20 @@
       <c r="B20" s="72" t="s">
         <v>170</v>
       </c>
-      <c r="C20" s="293">
-        <v>180486540.96000001</v>
-      </c>
-      <c r="D20" s="293" t="s">
-        <v>166</v>
-      </c>
-      <c r="E20" s="293" t="s">
-        <v>166</v>
-      </c>
-      <c r="F20" s="293">
+      <c r="C20" s="234">
+        <v>181076540.96000001</v>
+      </c>
+      <c r="D20" s="234">
+        <v>0</v>
+      </c>
+      <c r="E20" s="234">
+        <v>0</v>
+      </c>
+      <c r="F20" s="234">
         <v>10162161.880000001</v>
       </c>
-      <c r="G20" s="293">
-        <v>190648702.84</v>
+      <c r="G20" s="234">
+        <v>191238702.84</v>
       </c>
       <c r="H20" s="111"/>
       <c r="I20" s="111"/>
@@ -4099,27 +4099,27 @@
       <c r="B21" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="C21" s="293">
-        <v>370588155.39999998</v>
-      </c>
-      <c r="D21" s="293" t="s">
-        <v>166</v>
-      </c>
-      <c r="E21" s="293" t="s">
-        <v>166</v>
-      </c>
-      <c r="F21" s="293">
-        <v>14510450.060000001</v>
-      </c>
-      <c r="G21" s="293">
-        <v>385098605.45999998</v>
+      <c r="C21" s="234">
+        <v>394770155.39999998</v>
+      </c>
+      <c r="D21" s="234">
+        <v>0</v>
+      </c>
+      <c r="E21" s="234">
+        <v>0</v>
+      </c>
+      <c r="F21" s="234">
+        <v>16384323.880000001</v>
+      </c>
+      <c r="G21" s="234">
+        <v>411154479.27999997</v>
       </c>
       <c r="H21" s="111"/>
       <c r="I21" s="111"/>
       <c r="J21" s="111"/>
       <c r="M21" s="14">
         <f>SUM(C33,C34)+M20</f>
-        <v>668688076.87203598</v>
+        <v>706255031.93172801</v>
       </c>
       <c r="N21" s="10" t="s">
         <v>121</v>
@@ -4129,20 +4129,20 @@
       <c r="B22" s="72" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="293">
-        <v>226084854.50993201</v>
-      </c>
-      <c r="D22" s="293">
-        <v>37155880.779475003</v>
-      </c>
-      <c r="E22" s="293">
-        <v>119802793.27977499</v>
-      </c>
-      <c r="F22" s="293">
-        <v>412031182.91984499</v>
-      </c>
-      <c r="G22" s="293">
-        <v>795074711.48902702</v>
+      <c r="C22" s="234">
+        <v>253008958.53975001</v>
+      </c>
+      <c r="D22" s="234">
+        <v>42295988.919471003</v>
+      </c>
+      <c r="E22" s="234">
+        <v>129007973.439775</v>
+      </c>
+      <c r="F22" s="234">
+        <v>422380732.75984502</v>
+      </c>
+      <c r="G22" s="234">
+        <v>846693653.65884101</v>
       </c>
       <c r="H22" s="111"/>
       <c r="I22" s="111"/>
@@ -4152,20 +4152,20 @@
       <c r="B23" s="72" t="s">
         <v>125</v>
       </c>
-      <c r="C23" s="293">
-        <v>262177944.914325</v>
-      </c>
-      <c r="D23" s="293">
-        <v>72156108.32987</v>
-      </c>
-      <c r="E23" s="293">
-        <v>192502029.91870001</v>
-      </c>
-      <c r="F23" s="293">
-        <v>317536568.669429</v>
-      </c>
-      <c r="G23" s="293">
-        <v>844372651.83232403</v>
+      <c r="C23" s="234">
+        <v>296482384.99711603</v>
+      </c>
+      <c r="D23" s="234">
+        <v>76344627.269869998</v>
+      </c>
+      <c r="E23" s="234">
+        <v>196866894.838698</v>
+      </c>
+      <c r="F23" s="234">
+        <v>325392424.81942898</v>
+      </c>
+      <c r="G23" s="234">
+        <v>895086331.92511296</v>
       </c>
       <c r="H23" s="111"/>
       <c r="I23" s="111"/>
@@ -4175,20 +4175,20 @@
       <c r="B24" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="C24" s="293">
-        <v>362102305.36603498</v>
-      </c>
-      <c r="D24" s="293">
-        <v>47703495.530475996</v>
-      </c>
-      <c r="E24" s="293">
-        <v>183925416.61994201</v>
-      </c>
-      <c r="F24" s="293">
-        <v>555631019.66932297</v>
-      </c>
-      <c r="G24" s="293">
-        <v>1149362237.185776</v>
+      <c r="C24" s="234">
+        <v>386904925.25418103</v>
+      </c>
+      <c r="D24" s="234">
+        <v>53890954.970452003</v>
+      </c>
+      <c r="E24" s="234">
+        <v>190787984.24993801</v>
+      </c>
+      <c r="F24" s="234">
+        <v>606427416.90921795</v>
+      </c>
+      <c r="G24" s="234">
+        <v>1238011281.3837891</v>
       </c>
       <c r="H24" s="111"/>
       <c r="I24" s="111"/>
@@ -4198,20 +4198,20 @@
       <c r="B25" s="72" t="s">
         <v>184</v>
       </c>
-      <c r="C25" s="293">
-        <v>126788736.79275</v>
-      </c>
-      <c r="D25" s="293">
-        <v>87099277.234648004</v>
-      </c>
-      <c r="E25" s="293">
-        <v>149958830.11964101</v>
-      </c>
-      <c r="F25" s="293">
-        <v>54852170.700000003</v>
-      </c>
-      <c r="G25" s="293">
-        <v>418699014.84703898</v>
+      <c r="C25" s="234">
+        <v>129801367.359348</v>
+      </c>
+      <c r="D25" s="234">
+        <v>92258790.697632998</v>
+      </c>
+      <c r="E25" s="234">
+        <v>152757208.489638</v>
+      </c>
+      <c r="F25" s="234">
+        <v>55090008.539999999</v>
+      </c>
+      <c r="G25" s="234">
+        <v>429907375.08661902</v>
       </c>
       <c r="H25" s="111"/>
       <c r="I25" s="111"/>
@@ -4221,20 +4221,20 @@
       <c r="B26" s="72" t="s">
         <v>127</v>
       </c>
-      <c r="C26" s="293">
-        <v>285966720.96544099</v>
-      </c>
-      <c r="D26" s="293">
-        <v>202991187.37955901</v>
-      </c>
-      <c r="E26" s="293">
-        <v>287618874.64680499</v>
-      </c>
-      <c r="F26" s="293">
-        <v>16706594.929</v>
-      </c>
-      <c r="G26" s="293">
-        <v>793283377.92080498</v>
+      <c r="C26" s="234">
+        <v>296621622.48543602</v>
+      </c>
+      <c r="D26" s="234">
+        <v>204510362.406059</v>
+      </c>
+      <c r="E26" s="234">
+        <v>287992748.54679501</v>
+      </c>
+      <c r="F26" s="234">
+        <v>17193081.429000001</v>
+      </c>
+      <c r="G26" s="234">
+        <v>806317814.86729002</v>
       </c>
       <c r="H26" s="111"/>
       <c r="I26" s="111"/>
@@ -4276,8 +4276,8 @@
       <c r="B31" s="81" t="s">
         <v>131</v>
       </c>
-      <c r="C31" s="293">
-        <v>204377405.84914801</v>
+      <c r="C31" s="234">
+        <v>249028817.739032</v>
       </c>
       <c r="G31" s="111"/>
       <c r="H31" s="111"/>
@@ -4287,8 +4287,8 @@
       <c r="B32" s="81" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="293">
-        <v>363310835.80250001</v>
+      <c r="C32" s="234">
+        <v>374557187.54245001</v>
       </c>
       <c r="G32" s="111"/>
       <c r="H32" s="111"/>
@@ -4298,8 +4298,8 @@
       <c r="B33" s="81" t="s">
         <v>133</v>
       </c>
-      <c r="C33" s="293">
-        <v>127032122.82622001</v>
+      <c r="C33" s="234">
+        <v>136227366.02619001</v>
       </c>
       <c r="G33" s="111"/>
       <c r="H33" s="111"/>
@@ -4309,8 +4309,8 @@
       <c r="B34" s="81" t="s">
         <v>134</v>
       </c>
-      <c r="C34" s="293">
-        <v>540833954.04581594</v>
+      <c r="C34" s="234">
+        <v>569205665.90553796</v>
       </c>
       <c r="G34" s="111"/>
       <c r="H34" s="111"/>
@@ -4320,7 +4320,7 @@
       <c r="B35" s="81" t="s">
         <v>135</v>
       </c>
-      <c r="C35" s="293">
+      <c r="C35" s="234">
         <v>822000</v>
       </c>
       <c r="G35" s="111"/>
@@ -4355,17 +4355,17 @@
       </c>
     </row>
     <row r="40" spans="2:19" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B40" s="258" t="s">
+      <c r="B40" s="269" t="s">
         <v>222</v>
       </c>
-      <c r="C40" s="259"/>
-      <c r="D40" s="260"/>
+      <c r="C40" s="270"/>
+      <c r="D40" s="271"/>
       <c r="E40" s="66" t="s">
         <v>137</v>
       </c>
       <c r="F40" s="174">
         <f ca="1">IF(MONTH(TODAY())=8,DAY(TODAY())/DAY(EOMONTH(TODAY(),0)),IF(MONTH(TODAY())&gt;8,1,0))</f>
-        <v>0.77419354838709675</v>
+        <v>0.83870967741935487</v>
       </c>
       <c r="G40" s="192" t="s">
         <v>188</v>
@@ -4389,7 +4389,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="41" spans="2:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:19" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B41" s="68" t="s">
         <v>136</v>
       </c>
@@ -4452,35 +4452,35 @@
       </c>
       <c r="E42" s="46">
         <f>H65</f>
-        <v>3826874002.8409185</v>
+        <v>4054834363.3681707</v>
       </c>
       <c r="F42" s="176">
         <f>IFERROR(E42/D42,0)</f>
-        <v>0.77662065266732616</v>
+        <v>0.82288262101107801</v>
       </c>
       <c r="G42" s="184">
         <f>D42*$H$40-E42</f>
-        <v>1100723518.1590815</v>
+        <v>872763157.63182926</v>
       </c>
       <c r="H42" s="184">
         <f ca="1">IFERROR(G42/$C$3,0)</f>
-        <v>220144703.6318163</v>
+        <v>290921052.54394311</v>
       </c>
       <c r="I42" s="204">
         <f>D42*$J$40-E42</f>
-        <v>1100723518.1590815</v>
+        <v>872763157.63182926</v>
       </c>
       <c r="J42" s="204">
         <f ca="1">IFERROR(I42/$C$3,0)</f>
-        <v>220144703.6318163</v>
+        <v>290921052.54394311</v>
       </c>
       <c r="K42" s="185">
         <f>D42*$L$40-E42</f>
-        <v>1100723518.1590815</v>
+        <v>872763157.63182926</v>
       </c>
       <c r="L42" s="185">
         <f ca="1">IFERROR(K42/$C$3,0)</f>
-        <v>220144703.6318163</v>
+        <v>290921052.54394311</v>
       </c>
       <c r="S42" s="173">
         <v>0.8</v>
@@ -4499,35 +4499,35 @@
       </c>
       <c r="E43" s="46">
         <f>I65</f>
-        <v>851211453.41418207</v>
+        <v>895158901.87165999</v>
       </c>
       <c r="F43" s="176">
         <f>IFERROR(E43/D43,0)</f>
-        <v>0.65758898235036412</v>
+        <v>0.69153983885274495</v>
       </c>
       <c r="G43" s="184">
         <f>D43*$H$40-E43</f>
-        <v>443231544.05175745</v>
+        <v>399284095.59427953</v>
       </c>
       <c r="H43" s="184">
         <f ca="1">IFERROR(G43/$C$3,0)</f>
-        <v>88646308.810351491</v>
+        <v>133094698.5314265</v>
       </c>
       <c r="I43" s="204">
         <f>D43*$J$40-E43</f>
-        <v>443231544.05175745</v>
+        <v>399284095.59427953</v>
       </c>
       <c r="J43" s="204">
         <f ca="1">IFERROR(I43/$C$3,0)</f>
-        <v>88646308.810351491</v>
+        <v>133094698.5314265</v>
       </c>
       <c r="K43" s="185">
         <f>D43*$L$40-E43</f>
-        <v>443231544.05175745</v>
+        <v>399284095.59427953</v>
       </c>
       <c r="L43" s="185">
         <f ca="1">IFERROR(K43/$C$3,0)</f>
-        <v>88646308.810351491</v>
+        <v>133094698.5314265</v>
       </c>
       <c r="S43" s="173">
         <v>0.85</v>
@@ -4546,35 +4546,35 @@
       </c>
       <c r="E44" s="46">
         <f>J65</f>
-        <v>2335691612.2302098</v>
+        <v>2543765077.3437028</v>
       </c>
       <c r="F44" s="176">
         <f>IFERROR(E44/D44,0)</f>
-        <v>0.72622445657871293</v>
+        <v>0.79091965792261476</v>
       </c>
       <c r="G44" s="184">
         <f>IF(D44=0,0,D44*$H$40-E44)</f>
-        <v>880520112.76979017</v>
+        <v>672446647.65629721</v>
       </c>
       <c r="H44" s="184">
         <f ca="1">IFERROR(G44/$C$3,0)</f>
-        <v>176104022.55395803</v>
+        <v>224148882.55209908</v>
       </c>
       <c r="I44" s="204">
         <f>IF(D44=0,0,D44*$J$40-E44)</f>
-        <v>880520112.76979017</v>
+        <v>672446647.65629721</v>
       </c>
       <c r="J44" s="204">
         <f ca="1">IFERROR(I44/$C$3,0)</f>
-        <v>176104022.55395803</v>
+        <v>224148882.55209908</v>
       </c>
       <c r="K44" s="185">
         <f>IF(D44=0,0,D44*$L$40-E44)</f>
-        <v>880520112.76979017</v>
+        <v>672446647.65629721</v>
       </c>
       <c r="L44" s="185">
         <f ca="1">IFERROR(K44/$C$3,0)</f>
-        <v>176104022.55395803</v>
+        <v>224148882.55209908</v>
       </c>
       <c r="S44" s="173">
         <v>0.9</v>
@@ -4593,80 +4593,80 @@
       </c>
       <c r="E45" s="46">
         <f>SUM(C31,C32)+M21</f>
-        <v>1236376318.523684</v>
+        <v>1329841037.2132101</v>
       </c>
       <c r="F45" s="176">
         <f>IFERROR(E45/D45,0)</f>
-        <v>0.66259620262956831</v>
+        <v>0.71268561857492441</v>
       </c>
       <c r="G45" s="184">
         <f>D45*$H$40-E45</f>
-        <v>629581128.28482676</v>
+        <v>536116409.59530067</v>
       </c>
       <c r="H45" s="184">
         <f ca="1">IFERROR(G45/$C$3,0)</f>
-        <v>125916225.65696535</v>
+        <v>178705469.86510023</v>
       </c>
       <c r="I45" s="204">
         <f>D45*$J$40-E45</f>
-        <v>629581128.28482676</v>
+        <v>536116409.59530067</v>
       </c>
       <c r="J45" s="204">
         <f ca="1">IFERROR(I45/$C$3,0)</f>
-        <v>125916225.65696535</v>
+        <v>178705469.86510023</v>
       </c>
       <c r="K45" s="185">
         <f>D45*$L$40-E45</f>
-        <v>629581128.28482676</v>
+        <v>536116409.59530067</v>
       </c>
       <c r="L45" s="185">
         <f ca="1">IFERROR(K45/$C$3,0)</f>
-        <v>125916225.65696535</v>
+        <v>178705469.86510023</v>
       </c>
       <c r="S45" s="173">
         <v>0.95</v>
       </c>
     </row>
     <row r="46" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>SUM(D42:D45)</f>
         <v>11304209690.274448</v>
       </c>
       <c r="E46" s="47">
         <f>SUM(E42:E45)</f>
-        <v>8250153387.0089931</v>
+        <v>8823599379.7967453</v>
       </c>
       <c r="F46" s="177">
         <f>IFERROR(E46/D46,0)</f>
-        <v>0.72983017946906936</v>
+        <v>0.7805587141034821</v>
       </c>
       <c r="G46" s="181">
         <f>SUM(G42:G45)</f>
-        <v>3054056303.2654557</v>
+        <v>2480610310.4777069</v>
       </c>
       <c r="H46" s="181">
         <f ca="1">IFERROR(G46/$C$3,0)</f>
-        <v>610811260.65309119</v>
+        <v>826870103.49256897</v>
       </c>
       <c r="I46" s="186">
         <f>SUM(I42:I45)</f>
-        <v>3054056303.2654557</v>
+        <v>2480610310.4777069</v>
       </c>
       <c r="J46" s="186">
         <f ca="1">IFERROR(I46/$C$3,0)</f>
-        <v>610811260.65309119</v>
+        <v>826870103.49256897</v>
       </c>
       <c r="K46" s="186">
         <f>SUM(K42:K45)</f>
-        <v>3054056303.2654557</v>
+        <v>2480610310.4777069</v>
       </c>
       <c r="L46" s="186">
         <f ca="1">IFERROR(K46/$C$3,0)</f>
-        <v>610811260.65309119</v>
+        <v>826870103.49256897</v>
       </c>
       <c r="S46" s="173">
         <v>1</v>
@@ -4679,84 +4679,84 @@
       <c r="S47" s="173"/>
     </row>
     <row r="48" spans="2:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>214</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="262"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="273"/>
+      <c r="L48" s="283"/>
+      <c r="M48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="269"/>
-      <c r="Q48" s="269"/>
-      <c r="R48" s="270"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="261"/>
+      <c r="Q48" s="261"/>
+      <c r="R48" s="262"/>
     </row>
     <row r="49" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="286" t="s">
+      <c r="B49" s="284" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="286" t="s">
+      <c r="C49" s="284" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="253"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="287" t="s">
+      <c r="E49" s="254"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="255"/>
+      <c r="H49" s="285" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="288"/>
-      <c r="J49" s="288"/>
-      <c r="K49" s="289"/>
-      <c r="L49" s="290" t="s">
+      <c r="I49" s="286"/>
+      <c r="J49" s="286"/>
+      <c r="K49" s="287"/>
+      <c r="L49" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="M49" s="271" t="str">
+      <c r="M49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="N49" s="271" t="str">
+      <c r="N49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
-      <c r="O49" s="273" t="str">
+      <c r="O49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="P49" s="273" t="str">
+      <c r="P49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
-      <c r="Q49" s="275" t="str">
+      <c r="Q49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="R49" s="275" t="str">
+      <c r="R49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B50" s="267"/>
-      <c r="C50" s="267"/>
+      <c r="B50" s="259"/>
+      <c r="C50" s="259"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -4781,13 +4781,13 @@
       <c r="K50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="L50" s="291"/>
-      <c r="M50" s="272"/>
-      <c r="N50" s="272"/>
-      <c r="O50" s="274"/>
-      <c r="P50" s="274"/>
-      <c r="Q50" s="276"/>
-      <c r="R50" s="276"/>
+      <c r="L50" s="289"/>
+      <c r="M50" s="264"/>
+      <c r="N50" s="264"/>
+      <c r="O50" s="266"/>
+      <c r="P50" s="266"/>
+      <c r="Q50" s="268"/>
+      <c r="R50" s="268"/>
       <c r="T50" s="172" t="s">
         <v>217</v>
       </c>
@@ -4820,47 +4820,47 @@
       </c>
       <c r="H51" s="114" cm="1">
         <f t="array" ref="H51">SUM(SUMIF($B$10:$B$26,$T51:$U51,C$10:C$26))</f>
-        <v>226084854.50993201</v>
+        <v>253008958.53975001</v>
       </c>
       <c r="I51" s="114" cm="1">
         <f t="array" ref="I51">SUM(SUMIF($B$10:$B$26,$T51:$U51,D$10:D$26))</f>
-        <v>37155880.779475003</v>
+        <v>42295988.919471003</v>
       </c>
       <c r="J51" s="114" cm="1">
         <f t="array" ref="J51">SUM(SUMIF($B$10:$B$26,$T51:$U51,E$10:E$26))</f>
-        <v>119802793.27977499</v>
+        <v>129007973.439775</v>
       </c>
       <c r="K51" s="114">
         <f t="shared" ref="K51:K64" si="1">SUM(H51:J51)</f>
-        <v>383043528.56918204</v>
+        <v>424312920.898996</v>
       </c>
       <c r="L51" s="187">
         <f t="shared" ref="L51:L65" si="2">IFERROR(K51/G51,0)</f>
-        <v>0.67690504538359042</v>
+        <v>0.749835294309387</v>
       </c>
       <c r="M51" s="184">
         <f t="shared" ref="M51:M64" si="3">G51*$H$40-K51</f>
-        <v>182831303.03606606</v>
+        <v>141561910.7062521</v>
       </c>
       <c r="N51" s="184">
         <f t="shared" ref="N51:N65" ca="1" si="4">IFERROR(M51/$C$3,0)</f>
-        <v>36566260.607213214</v>
+        <v>47187303.568750702</v>
       </c>
       <c r="O51" s="180">
         <f t="shared" ref="O51:O64" si="5">G51*$J$40-K51</f>
-        <v>182831303.03606606</v>
+        <v>141561910.7062521</v>
       </c>
       <c r="P51" s="180">
         <f t="shared" ref="P51:P65" ca="1" si="6">IFERROR(O51/$C$3,0)</f>
-        <v>36566260.607213214</v>
+        <v>47187303.568750702</v>
       </c>
       <c r="Q51" s="185">
         <f t="shared" ref="Q51:Q64" si="7">G51*$L$40-K51</f>
-        <v>182831303.03606606</v>
+        <v>141561910.7062521</v>
       </c>
       <c r="R51" s="185">
         <f t="shared" ref="R51:R65" ca="1" si="8">IFERROR(Q51/$C$3,0)</f>
-        <v>36566260.607213214</v>
+        <v>47187303.568750702</v>
       </c>
       <c r="T51" t="s">
         <v>124</v>
@@ -4894,47 +4894,47 @@
       </c>
       <c r="H52" s="114" cm="1">
         <f t="array" ref="H52">SUM(SUMIF($B$10:$B$26,$T52:$U52,C$10:C$26))</f>
-        <v>191791371.05262703</v>
+        <v>206652112.07662702</v>
       </c>
       <c r="I52" s="114" cm="1">
         <f t="array" ref="I52">SUM(SUMIF($B$10:$B$26,$T52:$U52,D$10:D$26))</f>
-        <v>74860986.836649001</v>
+        <v>81600421.196626008</v>
       </c>
       <c r="J52" s="114" cm="1">
         <f t="array" ref="J52">SUM(SUMIF($B$10:$B$26,$T52:$U52,E$10:E$26))</f>
-        <v>336806453.01903105</v>
+        <v>356834291.18895</v>
       </c>
       <c r="K52" s="114">
         <f t="shared" si="1"/>
-        <v>603458810.90830708</v>
+        <v>645086824.46220303</v>
       </c>
       <c r="L52" s="187">
         <f t="shared" si="2"/>
-        <v>0.72095140020793325</v>
+        <v>0.77068432997389913</v>
       </c>
       <c r="M52" s="184">
         <f t="shared" si="3"/>
-        <v>233572382.50398183</v>
+        <v>191944368.95008588</v>
       </c>
       <c r="N52" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>46714476.500796363</v>
+        <v>63981456.316695295</v>
       </c>
       <c r="O52" s="180">
         <f t="shared" si="5"/>
-        <v>233572382.50398183</v>
+        <v>191944368.95008588</v>
       </c>
       <c r="P52" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>46714476.500796363</v>
+        <v>63981456.316695295</v>
       </c>
       <c r="Q52" s="185">
         <f t="shared" si="7"/>
-        <v>233572382.50398183</v>
+        <v>191944368.95008588</v>
       </c>
       <c r="R52" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>46714476.500796363</v>
+        <v>63981456.316695295</v>
       </c>
       <c r="T52" t="s">
         <v>70</v>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="H53" s="114" cm="1">
         <f t="array" ref="H53">SUM(SUMIF($B$10:$B$26,$T53:$U53,C$10:C$26))</f>
-        <v>180486540.96000001</v>
+        <v>181076540.96000001</v>
       </c>
       <c r="I53" s="114" cm="1">
         <f t="array" ref="I53">SUM(SUMIF($B$10:$B$26,$T53:$U53,D$10:D$26))</f>
@@ -4980,35 +4980,35 @@
       </c>
       <c r="K53" s="114">
         <f t="shared" si="1"/>
-        <v>180486540.96000001</v>
+        <v>181076540.96000001</v>
       </c>
       <c r="L53" s="187">
         <f t="shared" si="2"/>
-        <v>0.68638299958465976</v>
+        <v>0.68862674567010729</v>
       </c>
       <c r="M53" s="184">
         <f t="shared" si="3"/>
-        <v>82466564.039999992</v>
+        <v>81876564.039999992</v>
       </c>
       <c r="N53" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>16493312.807999998</v>
+        <v>27292188.013333332</v>
       </c>
       <c r="O53" s="180">
         <f t="shared" si="5"/>
-        <v>82466564.039999992</v>
+        <v>81876564.039999992</v>
       </c>
       <c r="P53" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>16493312.807999998</v>
+        <v>27292188.013333332</v>
       </c>
       <c r="Q53" s="185">
         <f t="shared" si="7"/>
-        <v>82466564.039999992</v>
+        <v>81876564.039999992</v>
       </c>
       <c r="R53" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>16493312.807999998</v>
+        <v>27292188.013333332</v>
       </c>
       <c r="T53" t="s">
         <v>170</v>
@@ -5042,47 +5042,47 @@
       </c>
       <c r="H54" s="114" cm="1">
         <f t="array" ref="H54">SUM(SUMIF($B$10:$B$26,$T54:$U54,C$10:C$26))</f>
-        <v>687162604.17452097</v>
+        <v>707734634.90601301</v>
       </c>
       <c r="I54" s="114" cm="1">
         <f t="array" ref="I54">SUM(SUMIF($B$10:$B$26,$T54:$U54,D$10:D$26))</f>
-        <v>25975566.479871999</v>
+        <v>27756665.599851999</v>
       </c>
       <c r="J54" s="114" cm="1">
         <f t="array" ref="J54">SUM(SUMIF($B$10:$B$26,$T54:$U54,E$10:E$26))</f>
-        <v>136407063.156075</v>
+        <v>154753955.22001499</v>
       </c>
       <c r="K54" s="114">
         <f t="shared" si="1"/>
-        <v>849545233.81046796</v>
+        <v>890245255.72587991</v>
       </c>
       <c r="L54" s="187">
         <f t="shared" si="2"/>
-        <v>1.0917091076123655</v>
+        <v>1.1440107189177278</v>
       </c>
       <c r="M54" s="184">
         <f t="shared" si="3"/>
-        <v>-71366112.754607916</v>
+        <v>-112066134.67001987</v>
       </c>
       <c r="N54" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>-14273222.550921584</v>
+        <v>-37355378.223339953</v>
       </c>
       <c r="O54" s="180">
         <f t="shared" si="5"/>
-        <v>-71366112.754607916</v>
+        <v>-112066134.67001987</v>
       </c>
       <c r="P54" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>-14273222.550921584</v>
+        <v>-37355378.223339953</v>
       </c>
       <c r="Q54" s="185">
         <f t="shared" si="7"/>
-        <v>-71366112.754607916</v>
+        <v>-112066134.67001987</v>
       </c>
       <c r="R54" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>-14273222.550921584</v>
+        <v>-37355378.223339953</v>
       </c>
       <c r="T54" t="s">
         <v>115</v>
@@ -5124,39 +5124,39 @@
       </c>
       <c r="J55" s="114">
         <f>E12</f>
-        <v>233585586.67908999</v>
+        <v>305207208.67878997</v>
       </c>
       <c r="K55" s="114">
         <f t="shared" si="1"/>
-        <v>254622441.09908798</v>
+        <v>326244063.09878796</v>
       </c>
       <c r="L55" s="187">
         <f t="shared" si="2"/>
-        <v>0.46218747883664141</v>
+        <v>0.5921941536581673</v>
       </c>
       <c r="M55" s="184">
         <f t="shared" si="3"/>
-        <v>296284826.53176761</v>
+        <v>224663204.5320676</v>
       </c>
       <c r="N55" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>59256965.306353524</v>
+        <v>74887734.844022527</v>
       </c>
       <c r="O55" s="180">
         <f t="shared" si="5"/>
-        <v>296284826.53176761</v>
+        <v>224663204.5320676</v>
       </c>
       <c r="P55" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>59256965.306353524</v>
+        <v>74887734.844022527</v>
       </c>
       <c r="Q55" s="185">
         <f t="shared" si="7"/>
-        <v>296284826.53176761</v>
+        <v>224663204.5320676</v>
       </c>
       <c r="R55" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>59256965.306353524</v>
+        <v>74887734.844022527</v>
       </c>
       <c r="T55" t="s">
         <v>220</v>
@@ -5190,47 +5190,47 @@
       </c>
       <c r="H56" s="114" cm="1">
         <f t="array" ref="H56">SUM(SUMIF($B$10:$B$26,$T56:$U56,C$10:C$26))</f>
-        <v>126788736.79275</v>
+        <v>129801367.359348</v>
       </c>
       <c r="I56" s="114" cm="1">
         <f t="array" ref="I56">SUM(SUMIF($B$10:$B$26,$T56:$U56,D$10:D$26))</f>
-        <v>87099277.234648004</v>
+        <v>92258790.697632998</v>
       </c>
       <c r="J56" s="114" cm="1">
         <f t="array" ref="J56">SUM(SUMIF($B$10:$B$26,$T56:$U56,E$10:E$26))</f>
-        <v>149958830.11964101</v>
+        <v>152757208.489638</v>
       </c>
       <c r="K56" s="114">
         <f t="shared" si="1"/>
-        <v>363846844.147039</v>
+        <v>374817366.546619</v>
       </c>
       <c r="L56" s="187">
         <f t="shared" si="2"/>
-        <v>0.58080441649547321</v>
+        <v>0.59831653172592336</v>
       </c>
       <c r="M56" s="184">
         <f t="shared" si="3"/>
-        <v>262606457.19398969</v>
+        <v>251635934.79440969</v>
       </c>
       <c r="N56" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>52521291.438797936</v>
+        <v>83878644.931469902</v>
       </c>
       <c r="O56" s="180">
         <f t="shared" si="5"/>
-        <v>262606457.19398969</v>
+        <v>251635934.79440969</v>
       </c>
       <c r="P56" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>52521291.438797936</v>
+        <v>83878644.931469902</v>
       </c>
       <c r="Q56" s="185">
         <f t="shared" si="7"/>
-        <v>262606457.19398969</v>
+        <v>251635934.79440969</v>
       </c>
       <c r="R56" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>52521291.438797936</v>
+        <v>83878644.931469902</v>
       </c>
       <c r="T56" t="s">
         <v>184</v>
@@ -5264,47 +5264,47 @@
       </c>
       <c r="H57" s="114" cm="1">
         <f t="array" ref="H57">SUM(SUMIF($B$10:$B$26,$T57:$U57,C$10:C$26))</f>
-        <v>584747098.20811999</v>
+        <v>611345406.22811997</v>
       </c>
       <c r="I57" s="114" cm="1">
         <f t="array" ref="I57">SUM(SUMIF($B$10:$B$26,$T57:$U57,D$10:D$26))</f>
-        <v>68513920.019765005</v>
+        <v>74143784.859764993</v>
       </c>
       <c r="J57" s="114" cm="1">
         <f t="array" ref="J57">SUM(SUMIF($B$10:$B$26,$T57:$U57,E$10:E$26))</f>
-        <v>285862027.34951901</v>
+        <v>307286171.54949898</v>
       </c>
       <c r="K57" s="114">
         <f t="shared" si="1"/>
-        <v>939123045.57740402</v>
+        <v>992775362.63738394</v>
       </c>
       <c r="L57" s="187">
         <f t="shared" si="2"/>
-        <v>0.80910659278426822</v>
+        <v>0.85533103978917735</v>
       </c>
       <c r="M57" s="184">
         <f t="shared" si="3"/>
-        <v>221568331.74252105</v>
+        <v>167916014.68254113</v>
       </c>
       <c r="N57" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>44313666.348504208</v>
+        <v>55972004.89418038</v>
       </c>
       <c r="O57" s="180">
         <f t="shared" si="5"/>
-        <v>221568331.74252105</v>
+        <v>167916014.68254113</v>
       </c>
       <c r="P57" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>44313666.348504208</v>
+        <v>55972004.89418038</v>
       </c>
       <c r="Q57" s="185">
         <f t="shared" si="7"/>
-        <v>221568331.74252105</v>
+        <v>167916014.68254113</v>
       </c>
       <c r="R57" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>44313666.348504208</v>
+        <v>55972004.89418038</v>
       </c>
       <c r="T57" t="s">
         <v>120</v>
@@ -5338,47 +5338,47 @@
       </c>
       <c r="H58" s="114" cm="1">
         <f t="array" ref="H58">SUM(SUMIF($B$10:$B$26,$T58:$U58,C$10:C$26))</f>
-        <v>262177944.914325</v>
+        <v>296482384.99711603</v>
       </c>
       <c r="I58" s="114" cm="1">
         <f t="array" ref="I58">SUM(SUMIF($B$10:$B$26,$T58:$U58,D$10:D$26))</f>
-        <v>72156108.32987</v>
+        <v>76344627.269869998</v>
       </c>
       <c r="J58" s="114" cm="1">
         <f t="array" ref="J58">SUM(SUMIF($B$10:$B$26,$T58:$U58,E$10:E$26))</f>
-        <v>192502029.91870001</v>
+        <v>196866894.838698</v>
       </c>
       <c r="K58" s="114">
         <f t="shared" si="1"/>
-        <v>526836083.16289496</v>
+        <v>569693907.10568404</v>
       </c>
       <c r="L58" s="187">
         <f t="shared" si="2"/>
-        <v>0.79094044478336634</v>
+        <v>0.85528301245308258</v>
       </c>
       <c r="M58" s="184">
         <f t="shared" si="3"/>
-        <v>139252099.12394214</v>
+        <v>96394275.181153059</v>
       </c>
       <c r="N58" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>27850419.824788429</v>
+        <v>32131425.060384352</v>
       </c>
       <c r="O58" s="180">
         <f t="shared" si="5"/>
-        <v>139252099.12394214</v>
+        <v>96394275.181153059</v>
       </c>
       <c r="P58" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>27850419.824788429</v>
+        <v>32131425.060384352</v>
       </c>
       <c r="Q58" s="185">
         <f t="shared" si="7"/>
-        <v>139252099.12394214</v>
+        <v>96394275.181153059</v>
       </c>
       <c r="R58" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>27850419.824788429</v>
+        <v>32131425.060384352</v>
       </c>
       <c r="T58" t="s">
         <v>125</v>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="H59" s="114" cm="1">
         <f t="array" ref="H59">SUM(SUMIF($B$10:$B$26,$T59:$U59,C$10:C$26))</f>
-        <v>370588155.39999998</v>
+        <v>394770155.39999998</v>
       </c>
       <c r="I59" s="114" cm="1">
         <f t="array" ref="I59">SUM(SUMIF($B$10:$B$26,$T59:$U59,D$10:D$26))</f>
@@ -5424,35 +5424,35 @@
       </c>
       <c r="K59" s="114">
         <f t="shared" si="1"/>
-        <v>370588155.39999998</v>
+        <v>394770155.39999998</v>
       </c>
       <c r="L59" s="187">
         <f t="shared" si="2"/>
-        <v>0.83494625969024849</v>
+        <v>0.88942903297272558</v>
       </c>
       <c r="M59" s="184">
         <f t="shared" si="3"/>
-        <v>73258560.600000024</v>
+        <v>49076560.600000024</v>
       </c>
       <c r="N59" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>14651712.120000005</v>
+        <v>16358853.533333341</v>
       </c>
       <c r="O59" s="180">
         <f t="shared" si="5"/>
-        <v>73258560.600000024</v>
+        <v>49076560.600000024</v>
       </c>
       <c r="P59" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>14651712.120000005</v>
+        <v>16358853.533333341</v>
       </c>
       <c r="Q59" s="185">
         <f t="shared" si="7"/>
-        <v>73258560.600000024</v>
+        <v>49076560.600000024</v>
       </c>
       <c r="R59" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>14651712.120000005</v>
+        <v>16358853.533333341</v>
       </c>
       <c r="T59" t="s">
         <v>171</v>
@@ -5486,47 +5486,47 @@
       </c>
       <c r="H60" s="114">
         <f>C11</f>
-        <v>313831855.63549697</v>
+        <v>324305725.654459</v>
       </c>
       <c r="I60" s="114">
         <f>D11</f>
-        <v>71686173.307567</v>
+        <v>74140960.586657003</v>
       </c>
       <c r="J60" s="114">
         <f>E11</f>
-        <v>107095552.073377</v>
+        <v>111974290.83337</v>
       </c>
       <c r="K60" s="114">
         <f t="shared" si="1"/>
-        <v>492613581.01644099</v>
+        <v>510420977.07448602</v>
       </c>
       <c r="L60" s="187">
         <f t="shared" si="2"/>
-        <v>0.7810665004728593</v>
+        <v>0.80930112707997104</v>
       </c>
       <c r="M60" s="184">
         <f t="shared" si="3"/>
-        <v>138079939.59699166</v>
+        <v>120272543.53894663</v>
       </c>
       <c r="N60" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>27615987.91939833</v>
+        <v>40090847.84631554</v>
       </c>
       <c r="O60" s="180">
         <f t="shared" si="5"/>
-        <v>138079939.59699166</v>
+        <v>120272543.53894663</v>
       </c>
       <c r="P60" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>27615987.91939833</v>
+        <v>40090847.84631554</v>
       </c>
       <c r="Q60" s="185">
         <f t="shared" si="7"/>
-        <v>138079939.59699166</v>
+        <v>120272543.53894663</v>
       </c>
       <c r="R60" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>27615987.91939833</v>
+        <v>40090847.84631554</v>
       </c>
       <c r="T60" t="s">
         <v>221</v>
@@ -5560,47 +5560,47 @@
       </c>
       <c r="H61" s="114" cm="1">
         <f t="array" ref="H61">SUM(SUMIF($B$10:$B$26,$T61:$U61,C$10:C$26))</f>
-        <v>362102305.36603498</v>
+        <v>386904925.25418103</v>
       </c>
       <c r="I61" s="114" cm="1">
         <f t="array" ref="I61">SUM(SUMIF($B$10:$B$26,$T61:$U61,D$10:D$26))</f>
-        <v>47703495.530475996</v>
+        <v>53890954.970452003</v>
       </c>
       <c r="J61" s="114" cm="1">
         <f t="array" ref="J61">SUM(SUMIF($B$10:$B$26,$T61:$U61,E$10:E$26))</f>
-        <v>183925416.61994201</v>
+        <v>190787984.24993801</v>
       </c>
       <c r="K61" s="114">
         <f t="shared" si="1"/>
-        <v>593731217.51645303</v>
+        <v>631583864.47457099</v>
       </c>
       <c r="L61" s="187">
         <f t="shared" si="2"/>
-        <v>0.77298675859163457</v>
+        <v>0.82226763521230561</v>
       </c>
       <c r="M61" s="184">
         <f t="shared" si="3"/>
-        <v>174368896.64102447</v>
+        <v>136516249.68290651</v>
       </c>
       <c r="N61" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>34873779.328204893</v>
+        <v>45505416.560968839</v>
       </c>
       <c r="O61" s="180">
         <f t="shared" si="5"/>
-        <v>174368896.64102447</v>
+        <v>136516249.68290651</v>
       </c>
       <c r="P61" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>34873779.328204893</v>
+        <v>45505416.560968839</v>
       </c>
       <c r="Q61" s="185">
         <f t="shared" si="7"/>
-        <v>174368896.64102447</v>
+        <v>136516249.68290651</v>
       </c>
       <c r="R61" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>34873779.328204893</v>
+        <v>45505416.560968839</v>
       </c>
       <c r="T61" t="s">
         <v>126</v>
@@ -5634,47 +5634,47 @@
       </c>
       <c r="H62" s="114" cm="1">
         <f t="array" ref="H62">SUM(SUMIF($B$10:$B$26,$T62:$U62,C$10:C$26))</f>
-        <v>122025113.198008</v>
+        <v>148548971.92346001</v>
       </c>
       <c r="I62" s="114" cm="1">
         <f t="array" ref="I62">SUM(SUMIF($B$10:$B$26,$T62:$U62,D$10:D$26))</f>
-        <v>30987765.915591002</v>
+        <v>34675794.324588999</v>
       </c>
       <c r="J62" s="114" cm="1">
         <f t="array" ref="J62">SUM(SUMIF($B$10:$B$26,$T62:$U62,E$10:E$26))</f>
-        <v>187321413.78949499</v>
+        <v>201845017.44949499</v>
       </c>
       <c r="K62" s="114">
         <f t="shared" si="1"/>
-        <v>340334292.90309399</v>
+        <v>385069783.69754398</v>
       </c>
       <c r="L62" s="187">
         <f t="shared" si="2"/>
-        <v>0.64392546448631327</v>
+        <v>0.72856671953915519</v>
       </c>
       <c r="M62" s="184">
         <f t="shared" si="3"/>
-        <v>188196277.2842384</v>
+        <v>143460786.48978841</v>
       </c>
       <c r="N62" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>37639255.456847683</v>
+        <v>47820262.163262807</v>
       </c>
       <c r="O62" s="180">
         <f t="shared" si="5"/>
-        <v>188196277.2842384</v>
+        <v>143460786.48978841</v>
       </c>
       <c r="P62" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>37639255.456847683</v>
+        <v>47820262.163262807</v>
       </c>
       <c r="Q62" s="185">
         <f t="shared" si="7"/>
-        <v>188196277.2842384</v>
+        <v>143460786.48978841</v>
       </c>
       <c r="R62" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>37639255.456847683</v>
+        <v>47820262.163262807</v>
       </c>
       <c r="T62" t="s">
         <v>112</v>
@@ -5708,47 +5708,47 @@
       </c>
       <c r="H63" s="114" cm="1">
         <f t="array" ref="H63">SUM(SUMIF($B$10:$B$26,$T63:$U63,C$10:C$26))</f>
-        <v>285966720.96544099</v>
+        <v>296621622.48543602</v>
       </c>
       <c r="I63" s="114" cm="1">
         <f t="array" ref="I63">SUM(SUMIF($B$10:$B$26,$T63:$U63,D$10:D$26))</f>
-        <v>202991187.37955901</v>
+        <v>204510362.406059</v>
       </c>
       <c r="J63" s="114" cm="1">
         <f t="array" ref="J63">SUM(SUMIF($B$10:$B$26,$T63:$U63,E$10:E$26))</f>
-        <v>287618874.64680499</v>
+        <v>287992748.54679501</v>
       </c>
       <c r="K63" s="114">
         <f t="shared" si="1"/>
-        <v>776576782.99180508</v>
+        <v>789124733.43829</v>
       </c>
       <c r="L63" s="187">
         <f t="shared" si="2"/>
-        <v>0.75360588891826796</v>
+        <v>0.76578267498428332</v>
       </c>
       <c r="M63" s="184">
         <f t="shared" si="3"/>
-        <v>253904526.15309787</v>
+        <v>241356575.70661294</v>
       </c>
       <c r="N63" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>50780905.230619572</v>
+        <v>80452191.90220432</v>
       </c>
       <c r="O63" s="180">
         <f t="shared" si="5"/>
-        <v>253904526.15309787</v>
+        <v>241356575.70661294</v>
       </c>
       <c r="P63" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>50780905.230619572</v>
+        <v>80452191.90220432</v>
       </c>
       <c r="Q63" s="185">
         <f t="shared" si="7"/>
-        <v>253904526.15309787</v>
+        <v>241356575.70661294</v>
       </c>
       <c r="R63" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>50780905.230619572</v>
+        <v>80452191.90220432</v>
       </c>
       <c r="T63" t="s">
         <v>127</v>
@@ -5782,47 +5782,47 @@
       </c>
       <c r="H64" s="114" cm="1">
         <f t="array" ref="H64">SUM(SUMIF($B$10:$B$26,$T64:$U64,C$10:C$26))</f>
-        <v>109997278.243664</v>
+        <v>114458134.163663</v>
       </c>
       <c r="I64" s="114" cm="1">
         <f t="array" ref="I64">SUM(SUMIF($B$10:$B$26,$T64:$U64,D$10:D$26))</f>
-        <v>114167660.60071</v>
+        <v>115627120.040686</v>
       </c>
       <c r="J64" s="114" cm="1">
         <f t="array" ref="J64">SUM(SUMIF($B$10:$B$26,$T64:$U64,E$10:E$26))</f>
-        <v>114805571.57876</v>
+        <v>148451332.85874</v>
       </c>
       <c r="K64" s="114">
         <f t="shared" si="1"/>
-        <v>338970510.42313397</v>
+        <v>378536587.06308901</v>
       </c>
       <c r="L64" s="187">
         <f t="shared" si="2"/>
-        <v>0.576067382644468</v>
+        <v>0.6433084124999483</v>
       </c>
       <c r="M64" s="184">
         <f t="shared" si="3"/>
-        <v>249451123.28761661</v>
+        <v>209885046.64766157</v>
       </c>
       <c r="N64" s="184">
         <f t="shared" ca="1" si="4"/>
-        <v>49890224.657523319</v>
+        <v>69961682.215887189</v>
       </c>
       <c r="O64" s="180">
         <f t="shared" si="5"/>
-        <v>249451123.28761661</v>
+        <v>209885046.64766157</v>
       </c>
       <c r="P64" s="180">
         <f t="shared" ca="1" si="6"/>
-        <v>49890224.657523319</v>
+        <v>69961682.215887189</v>
       </c>
       <c r="Q64" s="185">
         <f t="shared" si="7"/>
-        <v>249451123.28761661</v>
+        <v>209885046.64766157</v>
       </c>
       <c r="R64" s="185">
         <f t="shared" ca="1" si="8"/>
-        <v>49890224.657523319</v>
+        <v>69961682.215887189</v>
       </c>
       <c r="T64" t="s">
         <v>122</v>
@@ -5854,47 +5854,47 @@
       </c>
       <c r="H65" s="135">
         <f t="shared" si="9"/>
-        <v>3826874002.8409185</v>
+        <v>4054834363.3681707</v>
       </c>
       <c r="I65" s="135">
         <f t="shared" si="9"/>
-        <v>851211453.41418207</v>
+        <v>895158901.87165999</v>
       </c>
       <c r="J65" s="135">
         <f t="shared" si="9"/>
-        <v>2335691612.2302098</v>
+        <v>2543765077.3437028</v>
       </c>
       <c r="K65" s="135">
         <f t="shared" si="9"/>
-        <v>7013777068.4853096</v>
+        <v>7493758342.5835333</v>
       </c>
       <c r="L65" s="189">
         <f t="shared" si="2"/>
-        <v>0.74312244338891409</v>
+        <v>0.79397733280241889</v>
       </c>
       <c r="M65" s="181">
         <f>SUM(M51:M64)</f>
-        <v>2424475174.9806299</v>
+        <v>1944493900.8824062</v>
       </c>
       <c r="N65" s="181">
         <f t="shared" ca="1" si="4"/>
-        <v>484895034.996126</v>
+        <v>648164633.62746871</v>
       </c>
       <c r="O65" s="181">
         <f>SUM(O51:O64)</f>
-        <v>2424475174.9806299</v>
+        <v>1944493900.8824062</v>
       </c>
       <c r="P65" s="181">
         <f t="shared" ca="1" si="6"/>
-        <v>484895034.996126</v>
+        <v>648164633.62746871</v>
       </c>
       <c r="Q65" s="186">
         <f>SUM(Q51:Q64)</f>
-        <v>2424475174.9806299</v>
+        <v>1944493900.8824062</v>
       </c>
       <c r="R65" s="186">
         <f t="shared" ca="1" si="8"/>
-        <v>484895034.996126</v>
+        <v>648164633.62746871</v>
       </c>
     </row>
     <row r="66" spans="2:21" x14ac:dyDescent="0.25">
@@ -5903,23 +5903,23 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:21" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="282" t="s">
+      <c r="B67" s="290" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="283"/>
-      <c r="D67" s="283"/>
-      <c r="E67" s="283"/>
-      <c r="F67" s="284"/>
-      <c r="G67" s="268" t="s">
+      <c r="C67" s="291"/>
+      <c r="D67" s="291"/>
+      <c r="E67" s="291"/>
+      <c r="F67" s="292"/>
+      <c r="G67" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="H67" s="269"/>
-      <c r="I67" s="269"/>
-      <c r="J67" s="269"/>
-      <c r="K67" s="269"/>
-      <c r="L67" s="270"/>
-    </row>
-    <row r="68" spans="2:21" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="H67" s="261"/>
+      <c r="I67" s="261"/>
+      <c r="J67" s="261"/>
+      <c r="K67" s="261"/>
+      <c r="L67" s="262"/>
+    </row>
+    <row r="68" spans="2:21" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
         <v>152</v>
       </c>
@@ -5979,35 +5979,35 @@
       </c>
       <c r="E69" s="114">
         <f>IFERROR(C31,0)</f>
-        <v>204377405.84914801</v>
+        <v>249028817.739032</v>
       </c>
       <c r="F69" s="187">
         <f t="shared" ref="F69:F74" si="10">IFERROR(E69/D69,0)</f>
-        <v>0.6855967616974098</v>
+        <v>0.83538270926696256</v>
       </c>
       <c r="G69" s="184">
         <f>D69*$H$40-E69</f>
-        <v>93724069.051561326</v>
+        <v>49072657.161677331</v>
       </c>
       <c r="H69" s="184">
         <f t="shared" ref="H69:H74" ca="1" si="11">IFERROR(G69/$C$3,0)</f>
-        <v>18744813.810312264</v>
+        <v>16357552.387225777</v>
       </c>
       <c r="I69" s="204">
         <f>D69*$J$40-E69</f>
-        <v>93724069.051561326</v>
+        <v>49072657.161677331</v>
       </c>
       <c r="J69" s="204">
         <f t="shared" ref="J69:J74" ca="1" si="12">IFERROR(I69/$C$3,0)</f>
-        <v>18744813.810312264</v>
+        <v>16357552.387225777</v>
       </c>
       <c r="K69" s="185">
         <f>D69*$L$40-E69</f>
-        <v>93724069.051561326</v>
+        <v>49072657.161677331</v>
       </c>
       <c r="L69" s="185">
         <f t="shared" ref="L69:L74" ca="1" si="13">IFERROR(K69/$C$3,0)</f>
-        <v>18744813.810312264</v>
+        <v>16357552.387225777</v>
       </c>
     </row>
     <row r="70" spans="2:21" x14ac:dyDescent="0.25">
@@ -6023,35 +6023,35 @@
       </c>
       <c r="E70" s="114">
         <f>IFERROR(C32,0)</f>
-        <v>363310835.80250001</v>
+        <v>374557187.54245001</v>
       </c>
       <c r="F70" s="187">
         <f t="shared" si="10"/>
-        <v>0.82308308485308157</v>
+        <v>0.84856176858959664</v>
       </c>
       <c r="G70" s="184">
         <f>D70*$H$40-E70</f>
-        <v>78091548.098209321</v>
+        <v>66845196.35825932</v>
       </c>
       <c r="H70" s="184">
         <f t="shared" ca="1" si="11"/>
-        <v>15618309.619641865</v>
+        <v>22281732.119419772</v>
       </c>
       <c r="I70" s="204">
         <f>D70*$J$40-E70</f>
-        <v>78091548.098209321</v>
+        <v>66845196.35825932</v>
       </c>
       <c r="J70" s="204">
         <f t="shared" ca="1" si="12"/>
-        <v>15618309.619641865</v>
+        <v>22281732.119419772</v>
       </c>
       <c r="K70" s="185">
         <f>D70*$L$40-E70</f>
-        <v>78091548.098209321</v>
+        <v>66845196.35825932</v>
       </c>
       <c r="L70" s="185">
         <f t="shared" ca="1" si="13"/>
-        <v>15618309.619641865</v>
+        <v>22281732.119419772</v>
       </c>
     </row>
     <row r="71" spans="2:21" x14ac:dyDescent="0.25">
@@ -6067,35 +6067,35 @@
       </c>
       <c r="E71" s="114">
         <f>M21+M7</f>
-        <v>668688076.87203598</v>
+        <v>706255031.93172801</v>
       </c>
       <c r="F71" s="187">
         <f t="shared" si="10"/>
-        <v>0.59362239509136872</v>
+        <v>0.6269721535365036</v>
       </c>
       <c r="G71" s="184">
         <f>D71*$H$40-E71</f>
-        <v>457765511.13505626</v>
+        <v>420198556.07536423</v>
       </c>
       <c r="H71" s="184">
         <f t="shared" ca="1" si="11"/>
-        <v>91553102.227011248</v>
+        <v>140066185.35845473</v>
       </c>
       <c r="I71" s="204">
         <f>D71*$J$40-E71</f>
-        <v>457765511.13505626</v>
+        <v>420198556.07536423</v>
       </c>
       <c r="J71" s="204">
         <f t="shared" ca="1" si="12"/>
-        <v>91553102.227011248</v>
+        <v>140066185.35845473</v>
       </c>
       <c r="K71" s="185">
         <f>D71*$L$40-E71</f>
-        <v>457765511.13505626</v>
+        <v>420198556.07536423</v>
       </c>
       <c r="L71" s="185">
         <f t="shared" ca="1" si="13"/>
-        <v>91553102.227011248</v>
+        <v>140066185.35845473</v>
       </c>
     </row>
     <row r="72" spans="2:21" hidden="1" x14ac:dyDescent="0.25">
@@ -6197,49 +6197,49 @@
       </c>
       <c r="E74" s="115">
         <f>SUM(E69:E73)</f>
-        <v>1236376318.523684</v>
+        <v>1329841037.2132101</v>
       </c>
       <c r="F74" s="177">
         <f t="shared" si="10"/>
-        <v>0.66259620262956831</v>
+        <v>0.71268561857492441</v>
       </c>
       <c r="G74" s="181">
         <f>SUM(G69:G73)</f>
-        <v>629581128.28482687</v>
+        <v>536116409.59530091</v>
       </c>
       <c r="H74" s="181">
         <f t="shared" ca="1" si="11"/>
-        <v>125916225.65696537</v>
+        <v>178705469.86510029</v>
       </c>
       <c r="I74" s="186">
         <f>SUM(I69:I73)</f>
-        <v>629581128.28482687</v>
+        <v>536116409.59530091</v>
       </c>
       <c r="J74" s="186">
         <f t="shared" ca="1" si="12"/>
-        <v>125916225.65696537</v>
+        <v>178705469.86510029</v>
       </c>
       <c r="K74" s="186">
         <f>SUM(K69:K73)</f>
-        <v>629581128.28482687</v>
+        <v>536116409.59530091</v>
       </c>
       <c r="L74" s="186">
         <f t="shared" ca="1" si="13"/>
-        <v>125916225.65696537</v>
+        <v>178705469.86510029</v>
       </c>
     </row>
     <row r="77" spans="2:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -6247,8 +6247,8 @@
       </c>
     </row>
     <row r="79" spans="2:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="D80" s="131" cm="1">
         <f t="array" ref="D80">SUM(SUMIF($B$10:$B$26,$T80:$U80,$F$10:$F$26))</f>
-        <v>412031182.91984499</v>
+        <v>422380732.75984502</v>
       </c>
       <c r="T80" t="str">
         <f t="shared" ref="T80:U93" si="14">T51</f>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="D81" s="132" cm="1">
         <f t="array" ref="D81">SUM(SUMIF($B$10:$B$26,$T81:$U81,$F$10:$F$26))</f>
-        <v>123327296.84</v>
+        <v>127435405.09</v>
       </c>
       <c r="T81" t="str">
         <f t="shared" si="14"/>
@@ -6328,7 +6328,7 @@
       </c>
       <c r="D83" s="131" cm="1">
         <f t="array" ref="D83">SUM(SUMIF($B$10:$B$26,$T83:$U83,$F$10:$F$26))</f>
-        <v>336341085.36982101</v>
+        <v>382338202.54978102</v>
       </c>
       <c r="T83" t="str">
         <f t="shared" si="14"/>
@@ -6346,9 +6346,9 @@
       <c r="C84" s="56" t="s">
         <v>191</v>
       </c>
-      <c r="D84" s="132" t="str">
+      <c r="D84" s="132">
         <f>F12</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="T84" t="str">
         <f t="shared" si="14"/>
@@ -6368,7 +6368,7 @@
       </c>
       <c r="D85" s="131" cm="1">
         <f t="array" ref="D85">SUM(SUMIF($B$10:$B$26,$T85:$U85,$F$10:$F$26))</f>
-        <v>54852170.700000003</v>
+        <v>55090008.539999999</v>
       </c>
       <c r="T85" t="str">
         <f t="shared" si="14"/>
@@ -6388,7 +6388,7 @@
       </c>
       <c r="D86" s="132" cm="1">
         <f t="array" ref="D86">SUM(SUMIF($B$10:$B$26,$T86:$U86,$F$10:$F$26))</f>
-        <v>1300038656.6399341</v>
+        <v>1342211628.6399341</v>
       </c>
       <c r="T86" t="str">
         <f t="shared" si="14"/>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="D87" s="131" cm="1">
         <f t="array" ref="D87">SUM(SUMIF($B$10:$B$26,$T87:$U87,$F$10:$F$26))</f>
-        <v>317536568.669429</v>
+        <v>325392424.81942898</v>
       </c>
       <c r="T87" t="str">
         <f t="shared" si="14"/>
@@ -6428,7 +6428,7 @@
       </c>
       <c r="D88" s="132" cm="1">
         <f t="array" ref="D88">SUM(SUMIF($B$10:$B$26,$T88:$U88,$F$10:$F$26))</f>
-        <v>14510450.060000001</v>
+        <v>16384323.880000001</v>
       </c>
       <c r="T88" t="str">
         <f t="shared" si="14"/>
@@ -6468,7 +6468,7 @@
       </c>
       <c r="D90" s="131" cm="1">
         <f t="array" ref="D90">SUM(SUMIF($B$10:$B$26,$T90:$U90,$F$10:$F$26))</f>
-        <v>555631019.66932297</v>
+        <v>606427416.90921795</v>
       </c>
       <c r="T90" t="str">
         <f t="shared" si="14"/>
@@ -6488,7 +6488,7 @@
       </c>
       <c r="D91" s="132" cm="1">
         <f t="array" ref="D91">SUM(SUMIF($B$10:$B$26,$T91:$U91,$F$10:$F$26))</f>
-        <v>146701033.86000001</v>
+        <v>158023556.22</v>
       </c>
       <c r="T91" t="str">
         <f t="shared" si="14"/>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="D92" s="131" cm="1">
         <f t="array" ref="D92">SUM(SUMIF($B$10:$B$26,$T92:$U92,$F$10:$F$26))</f>
-        <v>16706594.929</v>
+        <v>17193081.429000001</v>
       </c>
       <c r="T92" t="str">
         <f t="shared" si="14"/>
@@ -6528,7 +6528,7 @@
       </c>
       <c r="D93" s="132" cm="1">
         <f t="array" ref="D93">SUM(SUMIF($B$10:$B$26,$T93:$U93,$F$10:$F$26))</f>
-        <v>114098921.278</v>
+        <v>118704326.79799999</v>
       </c>
       <c r="T93" t="str">
         <f t="shared" si="14"/>
@@ -6546,11 +6546,17 @@
       <c r="C94" s="58"/>
       <c r="D94" s="120">
         <f>SUM(D80:D93)</f>
-        <v>3684434246.9553514</v>
+        <v>3864240373.6552067</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="G67:L67"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="M48:R48"/>
@@ -6565,12 +6571,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <conditionalFormatting sqref="L51:L64">
     <cfRule type="expression" dxfId="14" priority="1">
@@ -7199,11 +7199,11 @@
       </c>
     </row>
     <row r="40" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="258" t="s">
+      <c r="B40" s="269" t="s">
         <v>162</v>
       </c>
-      <c r="C40" s="259"/>
-      <c r="D40" s="260"/>
+      <c r="C40" s="270"/>
+      <c r="D40" s="271"/>
       <c r="E40" s="66" t="s">
         <v>137</v>
       </c>
@@ -7472,10 +7472,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>SUM(D42:D45)</f>
         <v>0</v>
@@ -7523,84 +7523,84 @@
       <c r="S47" s="173"/>
     </row>
     <row r="48" spans="2:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="262"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="273"/>
+      <c r="L48" s="283"/>
+      <c r="M48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="269"/>
-      <c r="Q48" s="269"/>
-      <c r="R48" s="270"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="261"/>
+      <c r="Q48" s="261"/>
+      <c r="R48" s="262"/>
     </row>
     <row r="49" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="286" t="s">
+      <c r="B49" s="284" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="286" t="s">
+      <c r="C49" s="284" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="253"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="287" t="s">
+      <c r="E49" s="254"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="255"/>
+      <c r="H49" s="285" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="288"/>
-      <c r="J49" s="288"/>
-      <c r="K49" s="289"/>
-      <c r="L49" s="290" t="s">
+      <c r="I49" s="286"/>
+      <c r="J49" s="286"/>
+      <c r="K49" s="287"/>
+      <c r="L49" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="M49" s="271" t="str">
+      <c r="M49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="N49" s="271" t="str">
+      <c r="N49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="O49" s="273" t="str">
+      <c r="O49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="P49" s="273" t="str">
+      <c r="P49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="Q49" s="275" t="str">
+      <c r="Q49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="R49" s="275" t="str">
+      <c r="R49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="267"/>
-      <c r="C50" s="267"/>
+      <c r="B50" s="259"/>
+      <c r="C50" s="259"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -7625,13 +7625,13 @@
       <c r="K50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="L50" s="291"/>
-      <c r="M50" s="272"/>
-      <c r="N50" s="272"/>
-      <c r="O50" s="274"/>
-      <c r="P50" s="274"/>
-      <c r="Q50" s="276"/>
-      <c r="R50" s="276"/>
+      <c r="L50" s="289"/>
+      <c r="M50" s="264"/>
+      <c r="N50" s="264"/>
+      <c r="O50" s="266"/>
+      <c r="P50" s="266"/>
+      <c r="Q50" s="268"/>
+      <c r="R50" s="268"/>
       <c r="T50" s="178" t="s">
         <v>217</v>
       </c>
@@ -8747,21 +8747,21 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:21" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="282" t="s">
+      <c r="B67" s="290" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="283"/>
-      <c r="D67" s="283"/>
-      <c r="E67" s="283"/>
-      <c r="F67" s="292"/>
-      <c r="G67" s="268" t="s">
+      <c r="C67" s="291"/>
+      <c r="D67" s="291"/>
+      <c r="E67" s="291"/>
+      <c r="F67" s="293"/>
+      <c r="G67" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="H67" s="269"/>
-      <c r="I67" s="269"/>
-      <c r="J67" s="269"/>
-      <c r="K67" s="269"/>
-      <c r="L67" s="270"/>
+      <c r="H67" s="261"/>
+      <c r="I67" s="261"/>
+      <c r="J67" s="261"/>
+      <c r="K67" s="261"/>
+      <c r="L67" s="262"/>
     </row>
     <row r="68" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -9075,17 +9075,17 @@
     <row r="75" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="77" spans="2:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -9093,8 +9093,8 @@
       </c>
     </row>
     <row r="79" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -9398,6 +9398,12 @@
     <row r="95" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="G67:L67"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="M48:R48"/>
@@ -9412,12 +9418,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <conditionalFormatting sqref="L51:L64">
     <cfRule type="expression" dxfId="11" priority="1">
@@ -10045,11 +10045,11 @@
       </c>
     </row>
     <row r="40" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="258" t="s">
+      <c r="B40" s="269" t="s">
         <v>164</v>
       </c>
-      <c r="C40" s="259"/>
-      <c r="D40" s="260"/>
+      <c r="C40" s="270"/>
+      <c r="D40" s="271"/>
       <c r="E40" s="66" t="s">
         <v>137</v>
       </c>
@@ -10318,10 +10318,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>SUM(D42:D45)</f>
         <v>0</v>
@@ -10369,84 +10369,84 @@
       <c r="S47" s="173"/>
     </row>
     <row r="48" spans="2:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="262"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="273"/>
+      <c r="L48" s="283"/>
+      <c r="M48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="269"/>
-      <c r="Q48" s="269"/>
-      <c r="R48" s="270"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="261"/>
+      <c r="Q48" s="261"/>
+      <c r="R48" s="262"/>
     </row>
     <row r="49" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="286" t="s">
+      <c r="B49" s="284" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="286" t="s">
+      <c r="C49" s="284" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="253"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="287" t="s">
+      <c r="E49" s="254"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="255"/>
+      <c r="H49" s="285" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="288"/>
-      <c r="J49" s="288"/>
-      <c r="K49" s="289"/>
-      <c r="L49" s="290" t="s">
+      <c r="I49" s="286"/>
+      <c r="J49" s="286"/>
+      <c r="K49" s="287"/>
+      <c r="L49" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="M49" s="271" t="str">
+      <c r="M49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="N49" s="271" t="str">
+      <c r="N49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="O49" s="273" t="str">
+      <c r="O49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="P49" s="273" t="str">
+      <c r="P49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="Q49" s="275" t="str">
+      <c r="Q49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="R49" s="275" t="str">
+      <c r="R49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="267"/>
-      <c r="C50" s="267"/>
+      <c r="B50" s="259"/>
+      <c r="C50" s="259"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -10471,13 +10471,13 @@
       <c r="K50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="L50" s="291"/>
-      <c r="M50" s="272"/>
-      <c r="N50" s="272"/>
-      <c r="O50" s="274"/>
-      <c r="P50" s="274"/>
-      <c r="Q50" s="276"/>
-      <c r="R50" s="276"/>
+      <c r="L50" s="289"/>
+      <c r="M50" s="264"/>
+      <c r="N50" s="264"/>
+      <c r="O50" s="266"/>
+      <c r="P50" s="266"/>
+      <c r="Q50" s="268"/>
+      <c r="R50" s="268"/>
       <c r="T50" s="178" t="s">
         <v>217</v>
       </c>
@@ -11593,21 +11593,21 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:21" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="282" t="s">
+      <c r="B67" s="290" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="283"/>
-      <c r="D67" s="283"/>
-      <c r="E67" s="283"/>
-      <c r="F67" s="292"/>
-      <c r="G67" s="268" t="s">
+      <c r="C67" s="291"/>
+      <c r="D67" s="291"/>
+      <c r="E67" s="291"/>
+      <c r="F67" s="293"/>
+      <c r="G67" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="H67" s="269"/>
-      <c r="I67" s="269"/>
-      <c r="J67" s="269"/>
-      <c r="K67" s="269"/>
-      <c r="L67" s="270"/>
+      <c r="H67" s="261"/>
+      <c r="I67" s="261"/>
+      <c r="J67" s="261"/>
+      <c r="K67" s="261"/>
+      <c r="L67" s="262"/>
     </row>
     <row r="68" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -11921,17 +11921,17 @@
     <row r="75" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="77" spans="2:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -11939,8 +11939,8 @@
       </c>
     </row>
     <row r="79" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -12244,6 +12244,12 @@
     <row r="95" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="G67:L67"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="M48:R48"/>
@@ -12258,12 +12264,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <conditionalFormatting sqref="L51:L64">
     <cfRule type="expression" dxfId="8" priority="1">
@@ -12891,11 +12891,11 @@
       </c>
     </row>
     <row r="40" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="258" t="s">
+      <c r="B40" s="269" t="s">
         <v>176</v>
       </c>
-      <c r="C40" s="259"/>
-      <c r="D40" s="260"/>
+      <c r="C40" s="270"/>
+      <c r="D40" s="271"/>
       <c r="E40" s="66" t="s">
         <v>137</v>
       </c>
@@ -13164,10 +13164,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>SUM(D42:D45)</f>
         <v>0</v>
@@ -13215,84 +13215,84 @@
       <c r="S47" s="173"/>
     </row>
     <row r="48" spans="2:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="262"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="273"/>
+      <c r="L48" s="283"/>
+      <c r="M48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="269"/>
-      <c r="Q48" s="269"/>
-      <c r="R48" s="270"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="261"/>
+      <c r="Q48" s="261"/>
+      <c r="R48" s="262"/>
     </row>
     <row r="49" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="286" t="s">
+      <c r="B49" s="284" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="286" t="s">
+      <c r="C49" s="284" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="253"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="287" t="s">
+      <c r="E49" s="254"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="255"/>
+      <c r="H49" s="285" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="288"/>
-      <c r="J49" s="288"/>
-      <c r="K49" s="289"/>
-      <c r="L49" s="290" t="s">
+      <c r="I49" s="286"/>
+      <c r="J49" s="286"/>
+      <c r="K49" s="287"/>
+      <c r="L49" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="M49" s="271" t="str">
+      <c r="M49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="N49" s="271" t="str">
+      <c r="N49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="O49" s="273" t="str">
+      <c r="O49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="P49" s="273" t="str">
+      <c r="P49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="Q49" s="275" t="str">
+      <c r="Q49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="R49" s="275" t="str">
+      <c r="R49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="267"/>
-      <c r="C50" s="267"/>
+      <c r="B50" s="259"/>
+      <c r="C50" s="259"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -13317,13 +13317,13 @@
       <c r="K50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="L50" s="291"/>
-      <c r="M50" s="272"/>
-      <c r="N50" s="272"/>
-      <c r="O50" s="274"/>
-      <c r="P50" s="274"/>
-      <c r="Q50" s="276"/>
-      <c r="R50" s="276"/>
+      <c r="L50" s="289"/>
+      <c r="M50" s="264"/>
+      <c r="N50" s="264"/>
+      <c r="O50" s="266"/>
+      <c r="P50" s="266"/>
+      <c r="Q50" s="268"/>
+      <c r="R50" s="268"/>
       <c r="T50" s="178" t="s">
         <v>217</v>
       </c>
@@ -14439,21 +14439,21 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:21" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="282" t="s">
+      <c r="B67" s="290" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="283"/>
-      <c r="D67" s="283"/>
-      <c r="E67" s="283"/>
-      <c r="F67" s="292"/>
-      <c r="G67" s="268" t="s">
+      <c r="C67" s="291"/>
+      <c r="D67" s="291"/>
+      <c r="E67" s="291"/>
+      <c r="F67" s="293"/>
+      <c r="G67" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="H67" s="269"/>
-      <c r="I67" s="269"/>
-      <c r="J67" s="269"/>
-      <c r="K67" s="269"/>
-      <c r="L67" s="270"/>
+      <c r="H67" s="261"/>
+      <c r="I67" s="261"/>
+      <c r="J67" s="261"/>
+      <c r="K67" s="261"/>
+      <c r="L67" s="262"/>
     </row>
     <row r="68" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -14767,17 +14767,17 @@
     <row r="75" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="77" spans="2:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -14785,8 +14785,8 @@
       </c>
     </row>
     <row r="79" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -15090,6 +15090,12 @@
     <row r="95" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="G67:L67"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="M48:R48"/>
@@ -15104,12 +15110,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <conditionalFormatting sqref="L51:L64">
     <cfRule type="expression" dxfId="5" priority="1">
@@ -15737,11 +15737,11 @@
       </c>
     </row>
     <row r="40" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="258" t="s">
+      <c r="B40" s="269" t="s">
         <v>178</v>
       </c>
-      <c r="C40" s="259"/>
-      <c r="D40" s="260"/>
+      <c r="C40" s="270"/>
+      <c r="D40" s="271"/>
       <c r="E40" s="66" t="s">
         <v>137</v>
       </c>
@@ -16010,10 +16010,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>SUM(D42:D45)</f>
         <v>0</v>
@@ -16061,84 +16061,84 @@
       <c r="S47" s="173"/>
     </row>
     <row r="48" spans="2:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="262"/>
-      <c r="L48" s="285"/>
-      <c r="M48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="273"/>
+      <c r="L48" s="283"/>
+      <c r="M48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="269"/>
-      <c r="Q48" s="269"/>
-      <c r="R48" s="270"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="261"/>
+      <c r="Q48" s="261"/>
+      <c r="R48" s="262"/>
     </row>
     <row r="49" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="286" t="s">
+      <c r="B49" s="284" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="286" t="s">
+      <c r="C49" s="284" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="253"/>
-      <c r="G49" s="254"/>
-      <c r="H49" s="287" t="s">
+      <c r="E49" s="254"/>
+      <c r="F49" s="254"/>
+      <c r="G49" s="255"/>
+      <c r="H49" s="285" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="288"/>
-      <c r="J49" s="288"/>
-      <c r="K49" s="289"/>
-      <c r="L49" s="290" t="s">
+      <c r="I49" s="286"/>
+      <c r="J49" s="286"/>
+      <c r="K49" s="287"/>
+      <c r="L49" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="M49" s="271" t="str">
+      <c r="M49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="N49" s="271" t="str">
+      <c r="N49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$40,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="O49" s="273" t="str">
+      <c r="O49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="P49" s="273" t="str">
+      <c r="P49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$40,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="Q49" s="275" t="str">
+      <c r="Q49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="R49" s="275" t="str">
+      <c r="R49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$40,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="267"/>
-      <c r="C50" s="267"/>
+      <c r="B50" s="259"/>
+      <c r="C50" s="259"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -16163,13 +16163,13 @@
       <c r="K50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="L50" s="291"/>
-      <c r="M50" s="272"/>
-      <c r="N50" s="272"/>
-      <c r="O50" s="274"/>
-      <c r="P50" s="274"/>
-      <c r="Q50" s="276"/>
-      <c r="R50" s="276"/>
+      <c r="L50" s="289"/>
+      <c r="M50" s="264"/>
+      <c r="N50" s="264"/>
+      <c r="O50" s="266"/>
+      <c r="P50" s="266"/>
+      <c r="Q50" s="268"/>
+      <c r="R50" s="268"/>
       <c r="T50" s="178" t="s">
         <v>217</v>
       </c>
@@ -17271,21 +17271,21 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:21" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="282" t="s">
+      <c r="B67" s="290" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="283"/>
-      <c r="D67" s="283"/>
-      <c r="E67" s="283"/>
-      <c r="F67" s="292"/>
-      <c r="G67" s="268" t="s">
+      <c r="C67" s="291"/>
+      <c r="D67" s="291"/>
+      <c r="E67" s="291"/>
+      <c r="F67" s="293"/>
+      <c r="G67" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="H67" s="269"/>
-      <c r="I67" s="269"/>
-      <c r="J67" s="269"/>
-      <c r="K67" s="269"/>
-      <c r="L67" s="270"/>
+      <c r="H67" s="261"/>
+      <c r="I67" s="261"/>
+      <c r="J67" s="261"/>
+      <c r="K67" s="261"/>
+      <c r="L67" s="262"/>
     </row>
     <row r="68" spans="2:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -17599,17 +17599,17 @@
     <row r="75" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="76" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="77" spans="2:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -17617,8 +17617,8 @@
       </c>
     </row>
     <row r="79" spans="2:21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -17922,6 +17922,12 @@
     <row r="95" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="G67:L67"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="M48:R48"/>
@@ -17936,12 +17942,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <conditionalFormatting sqref="L51:L64">
     <cfRule type="expression" dxfId="2" priority="1">
@@ -18048,10 +18048,10 @@
       <c r="AM1" s="20"/>
     </row>
     <row r="3" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B3" s="235" t="s">
+      <c r="B3" s="236" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="235"/>
+      <c r="C3" s="236"/>
       <c r="D3" s="17" t="s">
         <v>29</v>
       </c>
@@ -20088,13 +20088,13 @@
       </c>
     </row>
     <row r="29" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B29" s="237" t="s">
+      <c r="B29" s="238" t="s">
         <v>102</v>
       </c>
-      <c r="C29" s="237"/>
-      <c r="D29" s="237"/>
-      <c r="E29" s="237"/>
-      <c r="F29" s="237"/>
+      <c r="C29" s="238"/>
+      <c r="D29" s="238"/>
+      <c r="E29" s="238"/>
+      <c r="F29" s="238"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -20657,10 +20657,10 @@
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="242" t="s">
+      <c r="B44" s="243" t="s">
         <v>145</v>
       </c>
-      <c r="C44" s="243"/>
+      <c r="C44" s="244"/>
       <c r="D44" s="47">
         <f>D41+D42+D43</f>
         <v>10658901739</v>
@@ -20700,23 +20700,23 @@
       <c r="N46" s="97"/>
     </row>
     <row r="47" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="244" t="s">
+      <c r="B47" s="245" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="244" t="s">
+      <c r="C47" s="245" t="s">
         <v>42</v>
       </c>
-      <c r="D47" s="245" t="s">
+      <c r="D47" s="246" t="s">
         <v>137</v>
       </c>
-      <c r="E47" s="246"/>
-      <c r="F47" s="247"/>
+      <c r="E47" s="247"/>
+      <c r="F47" s="248"/>
       <c r="G47" s="98" t="s">
         <v>138</v>
       </c>
       <c r="H47" s="98"/>
       <c r="I47" s="98"/>
-      <c r="J47" s="244" t="s">
+      <c r="J47" s="245" t="s">
         <v>139</v>
       </c>
       <c r="K47" s="99" t="s">
@@ -20724,13 +20724,13 @@
       </c>
       <c r="L47" s="99"/>
       <c r="M47" s="99"/>
-      <c r="N47" s="241" t="s">
+      <c r="N47" s="242" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="48" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B48" s="244"/>
-      <c r="C48" s="244"/>
+      <c r="B48" s="245"/>
+      <c r="C48" s="245"/>
       <c r="D48" s="100" t="s">
         <v>149</v>
       </c>
@@ -20749,7 +20749,7 @@
       <c r="I48" s="100" t="s">
         <v>130</v>
       </c>
-      <c r="J48" s="244"/>
+      <c r="J48" s="245"/>
       <c r="K48" s="101" t="s">
         <v>142</v>
       </c>
@@ -20759,7 +20759,7 @@
       <c r="M48" s="101" t="s">
         <v>145</v>
       </c>
-      <c r="N48" s="241"/>
+      <c r="N48" s="242"/>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="50" t="s">
@@ -21436,15 +21436,15 @@
       </c>
     </row>
     <row r="63" spans="2:14" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B63" s="238" t="s">
+      <c r="B63" s="239" t="s">
         <v>144</v>
       </c>
-      <c r="C63" s="239"/>
-      <c r="D63" s="239"/>
-      <c r="E63" s="239"/>
-      <c r="F63" s="239"/>
-      <c r="G63" s="239"/>
-      <c r="H63" s="240"/>
+      <c r="C63" s="240"/>
+      <c r="D63" s="240"/>
+      <c r="E63" s="240"/>
+      <c r="F63" s="240"/>
+      <c r="G63" s="240"/>
+      <c r="H63" s="241"/>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B64" s="224" t="s">
@@ -22224,10 +22224,10 @@
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="242" t="s">
+      <c r="B44" s="243" t="s">
         <v>145</v>
       </c>
-      <c r="C44" s="243"/>
+      <c r="C44" s="244"/>
       <c r="D44" s="47">
         <f>D41+D42+D43</f>
         <v>9776434571</v>
@@ -22267,23 +22267,23 @@
       <c r="N46" s="97"/>
     </row>
     <row r="47" spans="2:14" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="244" t="s">
+      <c r="B47" s="245" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="244" t="s">
+      <c r="C47" s="245" t="s">
         <v>42</v>
       </c>
-      <c r="D47" s="245" t="s">
+      <c r="D47" s="246" t="s">
         <v>137</v>
       </c>
-      <c r="E47" s="246"/>
-      <c r="F47" s="247"/>
+      <c r="E47" s="247"/>
+      <c r="F47" s="248"/>
       <c r="G47" s="98" t="s">
         <v>138</v>
       </c>
       <c r="H47" s="98"/>
       <c r="I47" s="98"/>
-      <c r="J47" s="244" t="s">
+      <c r="J47" s="245" t="s">
         <v>139</v>
       </c>
       <c r="K47" s="99" t="s">
@@ -22291,13 +22291,13 @@
       </c>
       <c r="L47" s="99"/>
       <c r="M47" s="99"/>
-      <c r="N47" s="241" t="s">
+      <c r="N47" s="242" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="48" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B48" s="244"/>
-      <c r="C48" s="244"/>
+      <c r="B48" s="245"/>
+      <c r="C48" s="245"/>
       <c r="D48" s="100" t="s">
         <v>149</v>
       </c>
@@ -22316,7 +22316,7 @@
       <c r="I48" s="100" t="s">
         <v>130</v>
       </c>
-      <c r="J48" s="244"/>
+      <c r="J48" s="245"/>
       <c r="K48" s="101" t="s">
         <v>142</v>
       </c>
@@ -22326,7 +22326,7 @@
       <c r="M48" s="101" t="s">
         <v>145</v>
       </c>
-      <c r="N48" s="241"/>
+      <c r="N48" s="242"/>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="50" t="s">
@@ -23003,15 +23003,15 @@
       </c>
     </row>
     <row r="63" spans="2:14" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B63" s="238" t="s">
+      <c r="B63" s="239" t="s">
         <v>144</v>
       </c>
-      <c r="C63" s="239"/>
-      <c r="D63" s="239"/>
-      <c r="E63" s="239"/>
-      <c r="F63" s="239"/>
-      <c r="G63" s="239"/>
-      <c r="H63" s="240"/>
+      <c r="C63" s="240"/>
+      <c r="D63" s="240"/>
+      <c r="E63" s="240"/>
+      <c r="F63" s="240"/>
+      <c r="G63" s="240"/>
+      <c r="H63" s="241"/>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B64" s="224" t="s">
@@ -23943,10 +23943,10 @@
       <c r="N43" s="24"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B44" s="255" t="s">
+      <c r="B44" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C44" s="256"/>
+      <c r="C44" s="257"/>
       <c r="D44" s="47">
         <f>D41+D42+D43</f>
         <v>9764990416</v>
@@ -24011,23 +24011,23 @@
       <c r="Q46" s="48"/>
     </row>
     <row r="47" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="257" t="s">
+      <c r="B47" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="257" t="s">
+      <c r="C47" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="D47" s="252" t="s">
+      <c r="D47" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E47" s="253"/>
-      <c r="F47" s="254"/>
+      <c r="E47" s="254"/>
+      <c r="F47" s="255"/>
       <c r="G47" s="69" t="s">
         <v>138</v>
       </c>
       <c r="H47" s="69"/>
       <c r="I47" s="69"/>
-      <c r="J47" s="257" t="s">
+      <c r="J47" s="258" t="s">
         <v>139</v>
       </c>
       <c r="K47" s="35" t="s">
@@ -24035,13 +24035,13 @@
       </c>
       <c r="L47" s="35"/>
       <c r="M47" s="35"/>
-      <c r="N47" s="251" t="s">
+      <c r="N47" s="252" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="48" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B48" s="257"/>
-      <c r="C48" s="257"/>
+      <c r="B48" s="258"/>
+      <c r="C48" s="258"/>
       <c r="D48" s="70" t="s">
         <v>149</v>
       </c>
@@ -24060,7 +24060,7 @@
       <c r="I48" s="70" t="s">
         <v>130</v>
       </c>
-      <c r="J48" s="257"/>
+      <c r="J48" s="258"/>
       <c r="K48" s="34" t="s">
         <v>142</v>
       </c>
@@ -24070,7 +24070,7 @@
       <c r="M48" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="N48" s="251"/>
+      <c r="N48" s="252"/>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B49" s="50" t="s">
@@ -24762,15 +24762,15 @@
       <c r="N62" s="24"/>
     </row>
     <row r="63" spans="2:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="248" t="s">
+      <c r="B63" s="249" t="s">
         <v>144</v>
       </c>
-      <c r="C63" s="249"/>
-      <c r="D63" s="249"/>
-      <c r="E63" s="249"/>
-      <c r="F63" s="249"/>
-      <c r="G63" s="249"/>
-      <c r="H63" s="250"/>
+      <c r="C63" s="250"/>
+      <c r="D63" s="250"/>
+      <c r="E63" s="250"/>
+      <c r="F63" s="250"/>
+      <c r="G63" s="250"/>
+      <c r="H63" s="251"/>
       <c r="I63" s="24"/>
       <c r="J63" s="24"/>
       <c r="K63" s="24"/>
@@ -25720,11 +25720,11 @@
       </c>
     </row>
     <row r="41" spans="2:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="258" t="s">
+      <c r="B41" s="269" t="s">
         <v>179</v>
       </c>
-      <c r="C41" s="259"/>
-      <c r="D41" s="260"/>
+      <c r="C41" s="270"/>
+      <c r="D41" s="271"/>
       <c r="E41" s="66" t="s">
         <v>137</v>
       </c>
@@ -25945,10 +25945,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>D43+D44+D45</f>
         <v>9680534906.7669907</v>
@@ -25995,59 +25995,59 @@
       </c>
     </row>
     <row r="48" spans="2:19" s="139" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="L48" s="269"/>
-      <c r="M48" s="269"/>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="270"/>
+      <c r="L48" s="261"/>
+      <c r="M48" s="261"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="262"/>
       <c r="Q48"/>
       <c r="R48"/>
     </row>
     <row r="49" spans="2:18" s="139" customFormat="1" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="266" t="s">
+      <c r="B49" s="277" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="266" t="s">
+      <c r="C49" s="277" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="263" t="s">
+      <c r="D49" s="274" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="264"/>
-      <c r="F49" s="265"/>
+      <c r="E49" s="275"/>
+      <c r="F49" s="276"/>
       <c r="G49" s="140" t="s">
         <v>138</v>
       </c>
       <c r="H49" s="140"/>
       <c r="I49" s="140"/>
-      <c r="J49" s="263" t="s">
+      <c r="J49" s="274" t="s">
         <v>139</v>
       </c>
-      <c r="K49" s="271" t="str">
+      <c r="K49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="L49" s="271" t="str">
+      <c r="L49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="M49" s="273" t="str">
+      <c r="M49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>SELISIH
 95%</v>
@@ -26062,7 +26062,7 @@
         <v>SELISIH
 100%</v>
       </c>
-      <c r="P49" s="275" t="str">
+      <c r="P49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>PER HARI
 100%</v>
@@ -26071,8 +26071,8 @@
       <c r="R49"/>
     </row>
     <row r="50" spans="2:18" s="139" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="266"/>
-      <c r="C50" s="266"/>
+      <c r="B50" s="277"/>
+      <c r="C50" s="277"/>
       <c r="D50" s="141" t="s">
         <v>149</v>
       </c>
@@ -26091,13 +26091,13 @@
       <c r="I50" s="142" t="s">
         <v>130</v>
       </c>
-      <c r="J50" s="263"/>
-      <c r="K50" s="272"/>
-      <c r="L50" s="272"/>
-      <c r="M50" s="274"/>
+      <c r="J50" s="274"/>
+      <c r="K50" s="264"/>
+      <c r="L50" s="264"/>
+      <c r="M50" s="266"/>
       <c r="N50" s="188"/>
       <c r="O50" s="183"/>
-      <c r="P50" s="276"/>
+      <c r="P50" s="268"/>
       <c r="Q50"/>
       <c r="R50"/>
     </row>
@@ -27031,19 +27031,19 @@
     </row>
     <row r="67" spans="1:19" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="139"/>
-      <c r="B67" s="248" t="s">
+      <c r="B67" s="249" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="249"/>
-      <c r="D67" s="249"/>
-      <c r="E67" s="249"/>
-      <c r="F67" s="249"/>
-      <c r="G67" s="249"/>
-      <c r="H67" s="249"/>
-      <c r="I67" s="249"/>
-      <c r="J67" s="249"/>
-      <c r="K67" s="249"/>
-      <c r="L67" s="250"/>
+      <c r="C67" s="250"/>
+      <c r="D67" s="250"/>
+      <c r="E67" s="250"/>
+      <c r="F67" s="250"/>
+      <c r="G67" s="250"/>
+      <c r="H67" s="250"/>
+      <c r="I67" s="250"/>
+      <c r="J67" s="250"/>
+      <c r="K67" s="250"/>
+      <c r="L67" s="251"/>
       <c r="M67" s="139"/>
       <c r="N67" s="139"/>
       <c r="O67" s="139"/>
@@ -27428,20 +27428,20 @@
       <c r="I76"/>
     </row>
     <row r="77" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
       <c r="G77"/>
       <c r="H77"/>
       <c r="I77"/>
     </row>
     <row r="78" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -27452,8 +27452,8 @@
       <c r="I78"/>
     </row>
     <row r="79" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -27640,6 +27640,13 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="J49:J50"/>
     <mergeCell ref="B78:B79"/>
     <mergeCell ref="C78:C79"/>
     <mergeCell ref="K48:P48"/>
@@ -27649,13 +27656,6 @@
     <mergeCell ref="P49:P50"/>
     <mergeCell ref="B67:L67"/>
     <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="J49:J50"/>
   </mergeCells>
   <conditionalFormatting sqref="J51:J64">
     <cfRule type="expression" dxfId="26" priority="8">
@@ -28417,11 +28417,11 @@
       </c>
     </row>
     <row r="41" spans="2:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="277" t="s">
+      <c r="B41" s="278" t="s">
         <v>180</v>
       </c>
-      <c r="C41" s="278"/>
-      <c r="D41" s="279"/>
+      <c r="C41" s="279"/>
+      <c r="D41" s="280"/>
       <c r="E41" s="66" t="s">
         <v>137</v>
       </c>
@@ -28642,10 +28642,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>D43+D44+D45</f>
         <v>10097522879.624619</v>
@@ -28695,80 +28695,80 @@
       </c>
     </row>
     <row r="48" spans="2:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="L48" s="269"/>
-      <c r="M48" s="269"/>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="270"/>
+      <c r="L48" s="261"/>
+      <c r="M48" s="261"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="262"/>
     </row>
     <row r="49" spans="2:16" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="257" t="s">
+      <c r="B49" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="257" t="s">
+      <c r="C49" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="254"/>
+      <c r="E49" s="254"/>
+      <c r="F49" s="255"/>
       <c r="G49" s="112" t="s">
         <v>138</v>
       </c>
       <c r="H49" s="112"/>
       <c r="I49" s="112"/>
-      <c r="J49" s="252" t="s">
+      <c r="J49" s="253" t="s">
         <v>139</v>
       </c>
-      <c r="K49" s="271" t="str">
+      <c r="K49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="L49" s="271" t="str">
+      <c r="L49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="M49" s="273" t="str">
+      <c r="M49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="N49" s="273" t="str">
+      <c r="N49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="O49" s="275" t="str">
+      <c r="O49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="P49" s="275" t="str">
+      <c r="P49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:16" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="257"/>
-      <c r="C50" s="257"/>
+      <c r="B50" s="258"/>
+      <c r="C50" s="258"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -28787,13 +28787,13 @@
       <c r="I50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="J50" s="252"/>
-      <c r="K50" s="272"/>
-      <c r="L50" s="272"/>
-      <c r="M50" s="274"/>
-      <c r="N50" s="274"/>
-      <c r="O50" s="276"/>
-      <c r="P50" s="276"/>
+      <c r="J50" s="253"/>
+      <c r="K50" s="264"/>
+      <c r="L50" s="264"/>
+      <c r="M50" s="266"/>
+      <c r="N50" s="266"/>
+      <c r="O50" s="268"/>
+      <c r="P50" s="268"/>
     </row>
     <row r="51" spans="2:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="167" t="s">
@@ -29699,19 +29699,19 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:16" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="248" t="s">
+      <c r="B67" s="249" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="249"/>
-      <c r="D67" s="249"/>
-      <c r="E67" s="249"/>
-      <c r="F67" s="249"/>
-      <c r="G67" s="249"/>
-      <c r="H67" s="249"/>
-      <c r="I67" s="249"/>
-      <c r="J67" s="249"/>
-      <c r="K67" s="249"/>
-      <c r="L67" s="250"/>
+      <c r="C67" s="250"/>
+      <c r="D67" s="250"/>
+      <c r="E67" s="250"/>
+      <c r="F67" s="250"/>
+      <c r="G67" s="250"/>
+      <c r="H67" s="250"/>
+      <c r="I67" s="250"/>
+      <c r="J67" s="250"/>
+      <c r="K67" s="250"/>
+      <c r="L67" s="251"/>
     </row>
     <row r="68" spans="2:16" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -30023,17 +30023,17 @@
       </c>
     </row>
     <row r="77" spans="2:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -30041,8 +30041,8 @@
       </c>
     </row>
     <row r="79" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -30227,6 +30227,17 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="J49:J50"/>
+    <mergeCell ref="B67:L67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="N49:N50"/>
     <mergeCell ref="K48:P48"/>
     <mergeCell ref="K49:K50"/>
@@ -30234,17 +30245,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="J49:J50"/>
-    <mergeCell ref="B67:L67"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
   </mergeCells>
   <conditionalFormatting sqref="J51:J64">
     <cfRule type="expression" dxfId="23" priority="1">
@@ -31002,11 +31002,11 @@
       </c>
     </row>
     <row r="41" spans="2:19" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="258" t="s">
+      <c r="B41" s="269" t="s">
         <v>181</v>
       </c>
-      <c r="C41" s="259"/>
-      <c r="D41" s="260"/>
+      <c r="C41" s="270"/>
+      <c r="D41" s="271"/>
       <c r="E41" s="66" t="s">
         <v>137</v>
       </c>
@@ -31228,10 +31228,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>D43+D44+D45</f>
         <v>10899555455</v>
@@ -31281,80 +31281,80 @@
       </c>
     </row>
     <row r="48" spans="2:19" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="L48" s="269"/>
-      <c r="M48" s="269"/>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="270"/>
+      <c r="L48" s="261"/>
+      <c r="M48" s="261"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="262"/>
     </row>
     <row r="49" spans="2:16" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="257" t="s">
+      <c r="B49" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="257" t="s">
+      <c r="C49" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="254"/>
+      <c r="E49" s="254"/>
+      <c r="F49" s="255"/>
       <c r="G49" s="112" t="s">
         <v>138</v>
       </c>
       <c r="H49" s="112"/>
       <c r="I49" s="112"/>
-      <c r="J49" s="252" t="s">
+      <c r="J49" s="253" t="s">
         <v>139</v>
       </c>
-      <c r="K49" s="271" t="str">
+      <c r="K49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="L49" s="271" t="str">
+      <c r="L49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="M49" s="273" t="str">
+      <c r="M49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="N49" s="273" t="str">
+      <c r="N49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="O49" s="275" t="str">
+      <c r="O49" s="267" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="P49" s="275" t="str">
+      <c r="P49" s="267" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="257"/>
-      <c r="C50" s="257"/>
+      <c r="B50" s="258"/>
+      <c r="C50" s="258"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -31373,13 +31373,13 @@
       <c r="I50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="J50" s="252"/>
-      <c r="K50" s="272"/>
-      <c r="L50" s="272"/>
-      <c r="M50" s="274"/>
-      <c r="N50" s="274"/>
-      <c r="O50" s="276"/>
-      <c r="P50" s="276"/>
+      <c r="J50" s="253"/>
+      <c r="K50" s="264"/>
+      <c r="L50" s="264"/>
+      <c r="M50" s="266"/>
+      <c r="N50" s="266"/>
+      <c r="O50" s="268"/>
+      <c r="P50" s="268"/>
     </row>
     <row r="51" spans="2:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="50" t="s">
@@ -32285,19 +32285,19 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:16" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="248" t="s">
+      <c r="B67" s="249" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="249"/>
-      <c r="D67" s="249"/>
-      <c r="E67" s="249"/>
-      <c r="F67" s="249"/>
-      <c r="G67" s="249"/>
-      <c r="H67" s="249"/>
-      <c r="I67" s="249"/>
-      <c r="J67" s="249"/>
-      <c r="K67" s="249"/>
-      <c r="L67" s="250"/>
+      <c r="C67" s="250"/>
+      <c r="D67" s="250"/>
+      <c r="E67" s="250"/>
+      <c r="F67" s="250"/>
+      <c r="G67" s="250"/>
+      <c r="H67" s="250"/>
+      <c r="I67" s="250"/>
+      <c r="J67" s="250"/>
+      <c r="K67" s="250"/>
+      <c r="L67" s="251"/>
     </row>
     <row r="68" spans="2:16" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -32609,17 +32609,17 @@
       </c>
     </row>
     <row r="77" spans="2:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -32627,8 +32627,8 @@
       </c>
     </row>
     <row r="79" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -32800,6 +32800,17 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="D49:F49"/>
+    <mergeCell ref="J49:J50"/>
+    <mergeCell ref="B67:L67"/>
+    <mergeCell ref="B77:D77"/>
     <mergeCell ref="N49:N50"/>
     <mergeCell ref="K48:P48"/>
     <mergeCell ref="K49:K50"/>
@@ -32807,17 +32818,6 @@
     <mergeCell ref="M49:M50"/>
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="P49:P50"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="J49:J50"/>
-    <mergeCell ref="B67:L67"/>
-    <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
   </mergeCells>
   <conditionalFormatting sqref="J51:J64">
     <cfRule type="expression" dxfId="20" priority="1">
@@ -33596,11 +33596,11 @@
       </c>
     </row>
     <row r="41" spans="2:19" s="191" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="258" t="s">
+      <c r="B41" s="269" t="s">
         <v>190</v>
       </c>
-      <c r="C41" s="259"/>
-      <c r="D41" s="260"/>
+      <c r="C41" s="270"/>
+      <c r="D41" s="271"/>
       <c r="E41" s="66" t="s">
         <v>137</v>
       </c>
@@ -33822,10 +33822,10 @@
       </c>
     </row>
     <row r="46" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="B46" s="255" t="s">
+      <c r="B46" s="256" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="256"/>
+      <c r="C46" s="257"/>
       <c r="D46" s="47">
         <f>D43+D44+D45</f>
         <v>11281613287.225662</v>
@@ -33875,80 +33875,80 @@
       </c>
     </row>
     <row r="48" spans="2:19" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B48" s="261" t="s">
+      <c r="B48" s="272" t="s">
         <v>146</v>
       </c>
-      <c r="C48" s="262"/>
-      <c r="D48" s="262"/>
-      <c r="E48" s="262"/>
-      <c r="F48" s="262"/>
-      <c r="G48" s="262"/>
-      <c r="H48" s="262"/>
-      <c r="I48" s="262"/>
-      <c r="J48" s="262"/>
-      <c r="K48" s="268" t="s">
+      <c r="C48" s="273"/>
+      <c r="D48" s="273"/>
+      <c r="E48" s="273"/>
+      <c r="F48" s="273"/>
+      <c r="G48" s="273"/>
+      <c r="H48" s="273"/>
+      <c r="I48" s="273"/>
+      <c r="J48" s="273"/>
+      <c r="K48" s="260" t="s">
         <v>187</v>
       </c>
-      <c r="L48" s="269"/>
-      <c r="M48" s="269"/>
-      <c r="N48" s="269"/>
-      <c r="O48" s="269"/>
-      <c r="P48" s="270"/>
+      <c r="L48" s="261"/>
+      <c r="M48" s="261"/>
+      <c r="N48" s="261"/>
+      <c r="O48" s="261"/>
+      <c r="P48" s="262"/>
     </row>
     <row r="49" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B49" s="257" t="s">
+      <c r="B49" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="257" t="s">
+      <c r="C49" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="D49" s="252" t="s">
+      <c r="D49" s="253" t="s">
         <v>137</v>
       </c>
-      <c r="E49" s="253"/>
-      <c r="F49" s="254"/>
+      <c r="E49" s="254"/>
+      <c r="F49" s="255"/>
       <c r="G49" s="112" t="s">
         <v>138</v>
       </c>
       <c r="H49" s="112"/>
       <c r="I49" s="112"/>
-      <c r="J49" s="252" t="s">
+      <c r="J49" s="253" t="s">
         <v>139</v>
       </c>
-      <c r="K49" s="271" t="str">
+      <c r="K49" s="263" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>SELISIH
 90%</v>
       </c>
-      <c r="L49" s="271" t="str">
+      <c r="L49" s="263" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($H$41,"0%")</f>
         <v>PER HARI
 90%</v>
       </c>
-      <c r="M49" s="273" t="str">
+      <c r="M49" s="265" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>SELISIH
 95%</v>
       </c>
-      <c r="N49" s="273" t="str">
+      <c r="N49" s="265" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($J$41,"0%")</f>
         <v>PER HARI
 95%</v>
       </c>
-      <c r="O49" s="280" t="str">
+      <c r="O49" s="281" t="str">
         <f>"SELISIH"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>SELISIH
 100%</v>
       </c>
-      <c r="P49" s="280" t="str">
+      <c r="P49" s="281" t="str">
         <f>"PER HARI"&amp;CHAR(10)&amp;TEXT($L$41,"0%")</f>
         <v>PER HARI
 100%</v>
       </c>
     </row>
     <row r="50" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B50" s="257"/>
-      <c r="C50" s="257"/>
+      <c r="B50" s="258"/>
+      <c r="C50" s="258"/>
       <c r="D50" s="70" t="s">
         <v>149</v>
       </c>
@@ -33967,13 +33967,13 @@
       <c r="I50" s="113" t="s">
         <v>130</v>
       </c>
-      <c r="J50" s="252"/>
-      <c r="K50" s="272"/>
-      <c r="L50" s="272"/>
-      <c r="M50" s="274"/>
-      <c r="N50" s="274"/>
-      <c r="O50" s="281"/>
-      <c r="P50" s="281"/>
+      <c r="J50" s="253"/>
+      <c r="K50" s="264"/>
+      <c r="L50" s="264"/>
+      <c r="M50" s="266"/>
+      <c r="N50" s="266"/>
+      <c r="O50" s="282"/>
+      <c r="P50" s="282"/>
     </row>
     <row r="51" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B51" s="50" t="s">
@@ -34879,19 +34879,19 @@
       <c r="I66" s="111"/>
     </row>
     <row r="67" spans="2:16" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="248" t="s">
+      <c r="B67" s="249" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="249"/>
-      <c r="D67" s="249"/>
-      <c r="E67" s="249"/>
-      <c r="F67" s="249"/>
-      <c r="G67" s="249"/>
-      <c r="H67" s="249"/>
-      <c r="I67" s="249"/>
-      <c r="J67" s="249"/>
-      <c r="K67" s="249"/>
-      <c r="L67" s="250"/>
+      <c r="C67" s="250"/>
+      <c r="D67" s="250"/>
+      <c r="E67" s="250"/>
+      <c r="F67" s="250"/>
+      <c r="G67" s="250"/>
+      <c r="H67" s="250"/>
+      <c r="I67" s="250"/>
+      <c r="J67" s="250"/>
+      <c r="K67" s="250"/>
+      <c r="L67" s="251"/>
     </row>
     <row r="68" spans="2:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
@@ -35203,17 +35203,17 @@
       </c>
     </row>
     <row r="77" spans="2:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="248" t="s">
+      <c r="B77" s="249" t="s">
         <v>172</v>
       </c>
-      <c r="C77" s="249"/>
-      <c r="D77" s="250"/>
+      <c r="C77" s="250"/>
+      <c r="D77" s="251"/>
     </row>
     <row r="78" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B78" s="267" t="s">
+      <c r="B78" s="259" t="s">
         <v>41</v>
       </c>
-      <c r="C78" s="267" t="s">
+      <c r="C78" s="259" t="s">
         <v>42</v>
       </c>
       <c r="D78" s="231" t="s">
@@ -35221,8 +35221,8 @@
       </c>
     </row>
     <row r="79" spans="2:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B79" s="257"/>
-      <c r="C79" s="257"/>
+      <c r="B79" s="258"/>
+      <c r="C79" s="258"/>
       <c r="D79" s="70" t="s">
         <v>169</v>
       </c>
@@ -35407,6 +35407,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B48:J48"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="C49:C50"/>
     <mergeCell ref="K48:P48"/>
     <mergeCell ref="B78:B79"/>
     <mergeCell ref="C78:C79"/>
@@ -35420,11 +35425,6 @@
     <mergeCell ref="N49:N50"/>
     <mergeCell ref="B67:L67"/>
     <mergeCell ref="B77:D77"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B48:J48"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="C49:C50"/>
   </mergeCells>
   <conditionalFormatting sqref="J51:J64">
     <cfRule type="expression" dxfId="17" priority="1">

</xml_diff>